<commit_message>
améliorations: eval ragas, read_chunks, ...
</commit_message>
<xml_diff>
--- a/ragas_data/ragas_results.xlsx
+++ b/ragas_data/ragas_results.xlsx
@@ -493,13 +493,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>["Requête exécutée: SELECT p.name, s.three_point_pct\nFROM stats s JOIN players p ON p.player_id = s.player_id\nWHERE s.season = '2024-25' AND s.three_points_attempted &gt;= 100\nORDER BY s.three_point_pct DESC LIMIT 1;\nRésultat: [('Seth Curry', 45.6)]"]</t>
+          <t>["Requête exécutée: SELECT p.name, s.three_point_pct\nFROM stats s JOIN players p ON p.player_id = s.player_id\nWHERE s.season = '2024-25' AND s.three_points_attempted &gt;= 100\nORDER BY s.three_point_pct DESC LIMIT 1;\nRésultat: [{'name': 'Seth Curry', 'three_point_pct': 45.6}]"]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Le joueur avec le meilleur pourcentage de réussite à 3 points sur la saison 2024-25, parmi ceux ayant tenté au moins 100 tirs à 3 points, est **Seth Curry** avec un taux de réussite de **45,6 %**.
-*Un tir à 3 points précis, mais une saison à suivre pour confirmer cette régularité.*</t>
+          <t>Le joueur avec le meilleur pourcentage de réussite à 3 points sur la saison 2024-25, parmi ceux ayant tenté au moins 100 tirs, est **Seth Curry** avec un taux de réussite de **45,6 %**.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -508,10 +507,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8426500874827111</v>
+        <v>0.8392584992535422</v>
       </c>
       <c r="G2" t="n">
         <v>0.9999999999</v>
@@ -520,11 +519,11 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8304107991636778</v>
+        <v>0.9828477140884069</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>chiffree</t>
+          <t>chiffrée</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -541,12 +540,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>["Requête exécutée: SELECT p.name, s.points\nFROM stats s JOIN players p ON p.player_id = s.player_id\nWHERE s.season = '2024-25'\nORDER BY s.points DESC LIMIT 1;\nRésultat: [('Shai Gilgeous-Alexander', 2485)]"]</t>
+          <t>["Requête exécutée: SELECT p.name, s.points\nFROM stats s JOIN players p ON p.player_id = s.player_id\nWHERE s.season = '2024-25'\nORDER BY s.points DESC LIMIT 1;\nRésultat: [{'name': 'Shai Gilgeous-Alexander', 'points': 2485}]"]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Le joueur ayant marqué le plus de points en saison régulière 2024-25 est **Shai Gilgeous-Alexander**, avec **2 485 points**.</t>
+          <t>Le joueur ayant marqué le plus de points en saison régulière 2024-25 est **Shai Gilgeous-Alexander**, avec un total de **2 485 points**.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -558,7 +557,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9367997962384166</v>
+        <v>0.9367185438412059</v>
       </c>
       <c r="G3" t="n">
         <v>0.9999999999</v>
@@ -567,11 +566,11 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0.7345157300142662</v>
+        <v>0.9843535792190152</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>chiffree</t>
+          <t>chiffrée</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -588,7 +587,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>["Requête exécutée: SELECT p.name, s.rebounds\nFROM stats s JOIN players p ON p.player_id = s.player_id\nWHERE s.season = '2024-25'\nORDER BY s.rebounds DESC LIMIT 1;\nRésultat: [('Ivica Zubac', 1008)]"]</t>
+          <t>["Requête exécutée: SELECT p.name, s.rebounds\nFROM stats s JOIN players p ON p.player_id = s.player_id\nWHERE s.season = '2024-25'\nORDER BY s.rebounds DESC LIMIT 1;\nRésultat: [{'name': 'Ivica Zubac', 'rebounds': 1008}]"]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -618,7 +617,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>chiffree</t>
+          <t>chiffrée</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -630,42 +629,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Quel joueur a le plus de passes décisives sur la saison ?</t>
+          <t>Quels sont les 3 meilleurs passeurs décisifs de la saison ?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>["Requête exécutée: SELECT p.name, s.assists\nFROM stats s JOIN players p ON p.player_id = s.player_id\nWHERE s.season = '2024-25'\nORDER BY s.assists DESC LIMIT 1;\nRésultat: [('Trae Young', 882)]"]</t>
+          <t>["Requête exécutée: SELECT p.name, s.assists\nFROM stats s JOIN players p ON p.player_id = s.player_id\nWHERE s.season = '2024-25'\nORDER BY s.assists DESC LIMIT 3;\nRésultat: [{'name': 'Trae Young', 'assists': 882}, {'name': 'Nikola Jokić', 'assists': 714}, {'name': 'James Harden', 'assists': 687}]"]</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Le joueur avec le plus de passes décisives lors de la saison 2024-25 est **Trae Young**, avec **882 passes** décisives.</t>
+          <t>Les trois meilleurs passeurs décisifs de la saison 2024-25 sont **Trae Young** (882 passes), **Nikola Jokić** (714 passes) et **James Harden** (687 passes). Une belle diversité de profils avec un meneur pur, un pivot polyvalent et un vétéran expérimenté.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Trae Young, avec 882 passes décisives sur la saison.</t>
+          <t>Trae Young, avec 882 passes décisives, suivi de Nikola Jokic avec 714 et de James Harden avec 687.</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7509395678875638</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.9999999999</v>
-      </c>
+        <v>0.822977103432613</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>0.9868541068152592</v>
+        <v>0.9031011220876446</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>chiffree</t>
+          <t>chiffrée</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -682,36 +679,33 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>['[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nPlayoff riser\nThe modern NBA being the most efficient NBA isn\'t just about rule changes; it\'s that too, but moreso it\'s offensive strategy centered around maximizing efficiency, and iMO players who are collectively more talented than ever. No reason why the player with the highest absolute Ts% shouldn\'t be considered the most efficient in history\n\nO Répondre\nGrenScrin ·-10j\nDefinitionof"mostefficientfirstoption"+rTs%\n\nO Repondre\nSad_Bathroom1448·-10j\nAgreed. I get why rTs% exists, but you wouldn\'t say the fastest computer in 1955 is the fastest computer ever just because it\'s so much faster than the average computer in 1955.\n\nO Repondre\ncostelci·-10j\nYou could argue it had the best engineering though, as it was the furthest ahead of the competition operating with the same technology. different eras matters in any way is up to you I guess.\n\nO Repondre\nMalcolmSupleX·-10j\nReggieTS%?\n\nO Repondre\nNiviclades·-10j\nRelative True Shooting is my guess\n\nO Repondre\nKawhi Leonard\n112\nStephen Curry\n4147\nJerry West\n4457\nKareemAbdul-Jabbar\n5762\nKevin Durant\n4985\nCharles Barkley\n2833\nDirk Nowitzki\n3663\nLeBron James\n8289\nShaquille O\'Neal\n5250\nWilt Chamberlain\n3607\nNikola Jokic\n2580\nMichael Jordan\n5987\nJames Harden\n3895\nHakeem Olajuwon\n3755\nJulius Erving\n4580\nTim Duncan\n5172\nDwyane Wade\n3954\nGiannis Antetokounmpo\n2270\nKobe Bryant\n5640\nLarry Bird\n3897\n\nO Repondre\npick-and-hoop·-10j\nWow, Kawhi was basically one or two playoff runs from passing Larry Bird, that is so unexpected.', "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\npick-and-hoop·-10j\nWow, Kawhi was basically one or two playoff runs from passing Larry Bird, that is so unexpected.\n\nO Repondre\ntheeExample· -10j\nWas? You know he's still playing right? Lol\n\nO Repondre\ncomposer_7 . -10j\nNice to see Charles Barkley here too. Most people think he was just rebounds like Dennis Rodman and not a great scorer too.\n\nO Repondre\nSerious-Question281 · -10j\nHe did score 8 points in 9 seconds once. Very efficient\n\nO Repondre\nTarrot469·-10j\nOne thing that stands out is how high Jerry West is without the 3-point line to help boost TS. And he's the best guard defender of his era. People massively sleep on him and he should be right on the top 10 border.\n\nO Repondre\nTorkzilla·-10j\nReggie was my favorite player growing up and I definitely think he can hang with just about any shooting\n\nO Repondre\nSterlingStRose·-10j\nMight be why he's in the hall of fame\n\nO Repondre\nben10toesdown ·-10j\nDWade is definitely ahead of Reggie.\n\nO Repondre\nGreedyWarlord · -10j\n3rd best SG of all time, arguably, top 5 definitely. Won 3 chips. One with a waning Shaq. That doesn't mean he was necessarily a more efficient scorer. there is an argument to say that Reggie may be the 5th most valuable guard for a single franchise ever after Jordan, Magic, Curry, and Kobe I'm just arguing this point. And after rereading it, Zeke is ahead of Reggie too\n\nO Repondre\ndjinngerale : -10j\ntop 5 definitely\nJordan, Kobe, Wade, Iverson and who else in your books?", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\nvmpafq· -10j\nIf you filter for Reggie's prime years you would have to do the same for the others to make a fair comparison. Most of these guys have double the volume at least.\n\nO Repondre\nEyeFar9259·-10j\nReggie has had one of the greatest playoff scoring peaks. So this follows\n\nO Repondre\nHendo8888·-10j\nHow does rTS% work?\n\nO Repondre\nvmpafq · -10j\nrelative to league average TS%Ithink\n\nO Repondre\nRecommendationReal61:-10j\nPoints 1 and 2 can be true, but don't provide enough to support the argument proposed in point 3. There are at least a dozen other guards who unlike Reggie actually won MVPs and/or Finals MVPs, so maybe\nefficiency isn't the most important statistic in measuring a guard's value.\n\nName me one player who comes close to 14 playoff series wins with zero HOF teammates in their prime.\n-2\n\nOk so from 1991 to 2002 when Reggie averaged 24PPG on 17 shots a game, who exactly do you think was the number one option?\nHe's not a better player than any of the 2o I listed, ofc not bc there is more to the game than efficient scoring. But he definitely was a first option, and his resume is absolutely top 50 material. He won a lot for someone who never had a superstar teammate.\n\nHow many does Butler have?", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\ndjinngerale : -10j\ntop 5 definitely\nJordan, Kobe, Wade, Iverson and who else in your books?\n\nO Repondre\nGreedyWarlord · -10j\nIt is pretty hard for me to choose the 5th one. Harden would be my choice, since I consider West a PG. Followed by Drexler and Gervin.\n\nO Repondre\nWhatever801 : -10j\nYeah Reggie is one of those guys where you have to really watch him to understand what he was like. Stats usually don't do it justice (well I guess this one does). Took the 98 bulls to 7.\n\nO Repondre\nJohnBlunt·-10j\nIt's funny because Reggie is probably the consensus worst player on this list\n\nO Repondre\nChrisclc13·-10j\nI think the most surprising take to me is that Larry Bird is at the bottom of this list.\n\nO Repondre\nwolfpack_57·-10j\nI wasn't around to watch, but wasn't he pretty reliant on screens to get open, and took less shots because he couldn't self-create? I think that takes away from the first option assertion because self creation should IMO be a part of first option status.\n\nO Repondre\ndevvinitely · -10j\nThis is why Ijoined this subreddit. I love this stuff\n\nO Repondre\nAcEr3_·-10j\nYeah Reggie is extremely underrated. Of course he's part of the top 75 but people do not truly understand fully how great Reggie was. I feel like over time more and more people are becoming aware which is good.", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nCRich19·-9j· Modifié il ya -9j\nThis is really cool, thank you! I've been trying to poke holes but really can't :)\nCouple guys to call out:\nKevin McHale, 3000+ playoff points, 115 rTS%, led in playoff points a couple years over Bird.\n·James Worthy, 3000+ playoff points, 107 rTS%, was the Lakers #1 scorer for majority of his career\n\nO Répondre\n\ndenimjeg · -10j\nBeing the most efficient relative to era &amp; actually being the most efficient are 2 different things\n\nO Repondre\n\nVirtual-Database-238 ·-10j\nI remember checking during the 2022-2023 season and AD had the highest playoff TS% ever, with Kawhi right behind him. I think that Gobert and Ayton have since played enough games to be counted and now they have the highest. What's AD's rTS?\n\nO Repondre\n\nhqppp A0 · -10j\nAD is at 110, across 1566 total playoff points. So really good, albeit smaller sample (plus debatable whether he's been the first option across these points given LeBron was neck and neck for the big 2020 run).\n\nORepondre\n\npick-and-hoop·-10j\nNaa, AD was the number 1 but LeBron has the popularity behind him. AD was unbelievable during their title run.\n\nO Répondre\n\nCurious_Teaching_683·-10j\nrefugee_man·-10j\nReggie wasn't what I'd really consider a first option. I believe Jalen Rose and Smits at various points had more shot attempts\n\nO Repondre", '[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nIcyAuthor1  -10j\nDidn\'t expect Bird, Giannis, and Duncan to be that low.\n\nrayrayiscray ·-10j\nGiannis I can understand, his ft% (and high volume of them) really brings down the overall ts%\neven despite being one of the most efficient 2pt scorers in league history.\n\nMarkoSeke·-10j\nTS rewards three point shooters. Also it\'s not "low", this is a list of the top of all time\n\nbigvahe33 ·-10j\nmchale was huge in the playoffs\n\nrajs1286·-10j\nDuncan has never been efficient, despite the narrative\n\nUnusual-Weather1902 ·-10j\nDidn\'t expect Kobe to be more efficient than Bird\n\nwvmothman · -10j\nThe equation must be wonky- no way Jordan would be this low.\n\nAkipella · -10j\nComm. du top 1%\nStill insane to see 6\'2" Steph where he is on these lists lol.\n\nCletus_Starfish · -10j\nI was really confused when OP said Kawhi was the only one who came close and didn\'t see his name anywhere near Reggie\'s. Had to look at it twice to even find him on there lol.\n\n107\n\nJWOLFBEARD·-10j\nKawhi is literally right next to Reggie. What\n\nBumbiedore ·-10j\nOP edited the post to sort the table\n\nCletus_Starfish · -9j\nWasn\'t originally. Thankfully OP edited the post, but it was in a seemingly totally random order before.\n\ngza_liquidswords·-10j\nI was confused until I saw Kawhai Leonard and Jerry West. In any case, I am not sure how rTs% is defined, but I do think this makes the case that Reggie is in stratosphere (playoff wise at least) with top 25 all time players.', "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\n\nPagelTheReal18·-10j\nI don't agree with you. But thanks for abusing the downvote button. And note, I did not and don't intend on EvER downvoting someone over a difference of opinion.\n\nO Repondre\n\nFalse_Pear1860·-10j\nWhat is this table sorted by?? Though it was crazy that Curry was so far down the list, but then realized he should be like 3rd place if sorted by rTS\n\nO Repondre\n\nAkipella ·-10j\nThey fixed it\n\nO Repondre\n\nZazi751·-10j\nIf you don't also provide how rTs is calculated then the whole list is garbage. Some of these guys played through multiple eras with significant shifts.\n\nO Repondre\n\njoeb1ow·-10j\nWow, I though DWade would be #1 seeing how he was gifted 503,244 free throws in the 2006 playoffs\n\nO Repondre\n\nNolofinwe_2782·-10j\nHe's one of the most overrated players of all time\nNow if he played in this era?25ppg probably\n\nO Repondre\n\nnotatowel420·-10j\nReggie is one of the most overrated players of all time. You remove that Knicks series he would be a forgotten player.\n\nO Repondre\n\nIcy-Role-6333 · -10j\nSo efficient he never won the playoffs.\n\nO Repondre\n\navd318.-7j\nReally illuminates how useless efficiency is as a metric\n\nO Repondre", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nGreedyWarlord · -10j\nThat's a solid #2 option\n\nchief_sitass · -10j\nI'm curious how for outside of the top 20 Karl Malone is\n\n---\n\nhqppp ·-10j\nHis career playoff rTS is 99 - which is pretty terrible for an all-time big man whose rTS is 109 in the regular season. I do not consider him a better playoff scorer than any of the 20 listed, personally.\n\n---\n\nnhthelegend ·-10j\nThe mailman doesn't deliver on Sunday's\n\nobk_74·-10j\nHe will make exceptions if his customers are a certain age though. The junior discount, if you will.\n\nNonKolobian ·-10j\nClassic Pippen\n\nbingbongninergong · -10j\nProbably about 13 spots\n\n3s2ng·-10j\nIt grinds my gear when I see data in a table that is not sorted logically.\n\nSportsBettingRef.-10j ·Modifié il ya-9j\nKawhi Leonard\t112\nStephen Curry\t4147\nJerry West\t4457\nKareemAbdul-Jabbar\t5762\nKevin Durant\t4985\nCharles Barkley\t2833\nDirk Nowitzki\t3663\nLeBron James\t8289\nShaquille O'Neal\t5250\nWilt Chamberlain\t3607\nNikola Jokic\t2580\nMichael Jordan\t5987\nJames Harden\t3895\nHakeem Olajuwon\t3755\nJulius Erving\t4580\nTim Duncan\t5172\nDwyane Wade\t3954\nGiannis Antetokounmpo\t2270\nKobe Bryant\t5640\nLarry Bird\t3897\n\n---\n\ndirtynashtyfilthy · -10j\nWhy'd you remove Dirk's 108?\n\nSportsBettingRef .-9j · Modifié il y a -9j\ndouble checking.\nEdit2.: I've correct it.\n\nIcyAuthor1  -10j\nDidn't expect Bird, Giannis, and Duncan to be that low.", '[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\n\navd318.-7j\nReally illuminates how useless efficiency is as a metric\n\nO Repondre\n\nimperialmoose · -10j\nInteresting little set of stats! Regarding that last sentence, you\'re not accounting for all sorts of parts of\nthe game. It would be foolish to base his ranking all time purely off one stat. But you could argue he\'s\ncrazy, he made all NBA 3 times. Part of that may have been playing in Indiana, but partly he also wasn\'t\nthat good. Of the NBA 75, he\'s definitely in the bottom 20.\n\n\nHe was that good in the playoffs. He was Jamal Murray on steroids in the he greatly increased his\noutput once the games mattered. You can\'t just look at his regular season accolades and use that as\nan argument. He was plain and simple an absolute monster in the playoffs.\n\n\nI remember, I was there. I don\'t have any issue with OP saying Miller was a great playoff riser - we\nknow! I was addressing the final statement OP made; that he was the 5th most valuable franchise\nguard ever. He simply wasn\'t. There was one season I tried to argue with my buddies that he was a\ntop 10 player in the league. Even that was seen as a stretch. Like, he was never in an MVP\ndiscussion or even close.\n\nIf the argument is "he stayed with Indiana for a really long time, so he overall was more valuable\nto Indiana than Wade was to Miami"...I guess? Maybe?', "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\n---\n\n[supprimé]\n\nOverall-Palpitation6·-10j·Modifié il y a-10j\nHe barely averaged 20 a game most years. He's like if Klay Thompson happened to be the Warriors' first option, on the same number of shot attempts.\n\ntrojan_man16·-10j\nGuy's prime was in the late 90s/early 2000s. That's the modern NBA's dead ball era. Even 18ppg was a big deal then, 20+ was actually impressive. With today's pace and a system optimizing his skills Reggie would be a 25ppg+ guy.\n\nMadpsu444·-10j\nReggie Miller is the most efficient first option in NBA playoff history\n\n---\n\nOverall-Palpitation6·-10j·Modifié il y a -10j\nFair enough, but even in his era, there were still 25-30ppg guys, and he was never one of them. Reggie finished top 10 in ppg once during his career, in 1989-90, when he finished 8th with 24.6ppg. Reggie never topped 26 USG%, and hovered in the low-to-mid 20s in USG% for his entire prime, so even if he was Indiana's de-facto #1 scorer, he really never got used or scored like a true #1, even in a lower possession era.\n\nvmpafq·-10j\nThat's cap. MJ, Shaq, Iverson types were averaging 30 then."]</t>
+          <t>["[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nBut feels like leaving out playoff ppg really takes away some important context\n(both Reggie n Kawhi avg less than 21.5, n aren't even in the top 60...)\n\nO Repondre\ndenimjeg · -10j\nBeing the most efficient relative to era &amp; actually being the most efficient are 2 different things\n\nO Repondre\nVirtual-Database-238 ·-10j\nI remember checking during the 2022-2023 season and AD had the highest playoff TS% ever, with Kawhi right behind him. I think that Gobert and Ayton have since played enough games to be counted and now they have the highest. What's AD's rTS?\n\nO Repondre\nhqppp A0 · -10j\nAD is at 110, across 1566 total playoff points. So really good, albeit smaller sample (plus debatable whether he's been the first option across these points given LeBron was neck and neck for the big 2020 run).\n\nORepondre\npick-and-hoop·-10j\nNaa, AD was the number 1 but LeBron has the popularity behind him. AD was unbelievable during their title run.", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nchief_sitass · -10j\nHis career playoff rTS is 99 - which is pretty terrible for an all-time big man whose rTS is 109 in the regular season. I do not consider him a better playoff scorer than any of the 2o listed, personally.\n\nnhthelegend ·-10j\nThe mailman doesn't deliver on Sunday's\n\nobk_74·-10j\nHe will make exceptions if his customers are a certain age though. The junior discount, if you will.\n\nNonKolobian ·-10j\nClassic Pippen\n\nbingbongninergong ·-10j\nProbably about 13 spots\n\n3s2ng·-10j\nIt grinds my gear when I see data in a table that is not sorted logically.\n\nSportsBettingRef.-10j ·Modifié il y a-9j\nKawhi Leonard\t112\nStephen Curry\t110\nJerry West\t110\nKareemAbdul-Jabbar\t109\nKevin Durant\t109\nCharles Barkley\t109\nDirk Nowitzki\t108\nLeBron James\t107\nShaquille O'Neal\t107\nWilt Chamberlain\t107\nNikola Jokic\t107\nMichael Jordan\t106\nJames Harden\t106\nHakeem Olajuwon\t106\nJulius Erving\t105\nTim Duncan\t104\nDwyane Wade\t103\nGiannis Antetokounmpo\t103\nKobe Bryant\t102\nLarry Bird\t102", '[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nGrenScrin ·-10j\nDefinitionof"mostefficientfirstoption"+rTs%\n\nSad_Bathroom1448·-10j\nAgreed. I get why rTs% exists, but you wouldn\'t say the fastest computer in 1955 is the fastest \ncomputer ever just because it\'s so much faster than the average computer in 1955.\n\ndifferent eras matters in any way is up to you I guess.\n\ncostelci·-10j\nYou could argue it had the best engineering ever though, as it was the furthest ahead of the \ncompetition operating with the same technology.\n\nMalcolmSupleX·-10j\nReggieTS%?\n\nNiviclades·-10j\nRelative True Shooting is my guess\n\nKawhi Leonard\n112\n\nStephen Curry\n4147\n\nJerry West\n4457\n110\n\nKareemAbdul-Jabbar\n5762\n109\n\nKevin Durant\n4985\n109\n\nCharles Barkley\n2833\n109\n\nDirk Nowitzki\n3663\n108\n\nLeBron James\n8289\n107\n\nShaquille O\'Neal\n5250\n107\n\nWilt Chamberlain\n3607\n107\n\nNikola Jokic\n2580\n107\n\nMichael Jordan\n5987\n106\n\nJames Harden\n3895\n106\n\nHakeem Olajuwon\n3755\n106\n\nJulius Erving\n4580\n105\n\nTim Duncan\n5172\n104\n\nDwyane Wade\n3954\n103\n\nGiannis Antetokounmpo\n2270\n103', "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nHe is also one of the worst announcers that somehow keeps getting work\n\nDo we have numbers when excluding the shorter 3pt line?\n6th most valuable guard. Don't forget Dwade was the only reason Miami has ANY rings. Hes the second, or third best 2 guard in history, depending on how you value Kobe.\n\nCRich19·-9j· Modifié il ya -9j\nThis is really cool, thank you! I've been trying to poke holes but really can't :)\nCouple guys to call out:\nKevin McHale, 3000+ playoff points, 115 rTS%, led in playoff points a couple years over Bird.\n·James Worthy, 3000+ playoff points, 107 rTS%, was the Lakers #1 scorer for majority of his career\n\nReggie Miller is the most efficient first option in NBA playoff history : r/nba\n\nBut feels like leaving out playoff ppg really takes away some important context\n(both Reggie n Kawhi avg less than 21.5, n aren't even in the top 60...)\n\nO Repondre\ndenimjeg · -10j\nBeing the most efficient relative to era &amp; actually being the most efficient are 2 different things", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nDirk Nowitzki\n3663\n108\n\nLeBron James\n8289\n107\n\nShaquille O'Neal\n5250\n107\n\nWilt Chamberlain\n3607\n107\n\nNikola Jokic\n2580\n107\n\nMichael Jordan\n5987\n106\n\nJames Harden\n3895\n106\n\nHakeem Olajuwon\n3755\n106\n\nJulius Erving\n4580\n105\n\nTim Duncan\n5172\n104\n\nDwyane Wade\n3954\n103\n\nGiannis Antetokounmpo\n2270\n103\n\nKobe Bryant\n5640\n102\n\nLarry Bird\n3897\n102\n\npick-and-hoop·-10j\nWow, Kawhi was basically one or two playoff runs from passing Larry Bird, that is so unexpected.\n\n\ntheeExample· -10j\nWas? You know he's still playing right? Lol\n\nNice to see Charles Barkley here too. Most people think he was just rebounds like Dennis Rodman and \nnot a great scorer too.\n\nSerious-Question281 · -10j\nHe did score 8 points in 9 seconds once. Very efficient\n\nTarrot469·-10j\nOne thing that stands out is how high Jerry West is without the 3-point line to help boost TS. And he's the \nbest guard defender of his era. People massively sleep on him and he should be right on the top 10 \nborder."]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>D'après les données disponibles dans le contexte fourni, **aucune information précise sur le pourcentage de réussite à 3 points des joueurs sur les 5 derniers matchs** n'est mentionnée.
-Les discussions du Reddit se concentrent principalement sur des statistiques de carrière (comme le *rTS%* ou *True Shooting Percentage* relatif) ou des performances en playoffs sur plusieurs saisons, mais **rien ne concerne les performances récentes en termes de pourcentage à 3 points**.
-**Réponse :**
-*"Les données nécessaires pour répondre à cette question (pourcentage de réussite à 3 points sur les 5 derniers matchs) ne sont pas disponibles dans la base de connaissances actuelle."*</t>
+          <t>Désolé, les infos ne sont pas disponibles dans la base de connaissances de ce RAG.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Information non disponible : les données ne contiennent que des statistiques agrégées sur la saison entière, sans détail match par match.</t>
+          <t>Désolé, les infos ne sont pas disponibles dans la base de connaissances de ce RAG.</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2666666666577778</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0.5440069905149583</v>
+        <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -732,22 +726,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>['[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n58 upvotes- 6 commentaires\nr/AllAmericanTV.il y a1a\nWhat NFL team will Spencer play for?\n\n25 upvotes : 19 commentaires\nr/nba · il y a 13 a\nNBA Court Explained\n\n25 upvotes : 19 commentaires\nr/nba· il ya6a\nCan someone explain to me what it means for a team in the playoffs to take home court?', "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n101 upvotes : 44 commentaires\nr/nba·il y a 11j\n[Smith] This is now reality. Thunder vs Pacers will be the first NBA Finals since the luxury tax has been in effect where neither team was a taxpayer for that season.\n\n11 k upvotes : 948 commentaires\nr/hockey · il y a 13j\nThe Oilers are the first Canadian team to have home-ice advantage in the Stanley Cup Finals since the 2011 Vancouver Canucks\n\n2,5 k upvotes : 226 commentaires\nr/nba·ilya 11j\nThe Knicks have now lost to a lower seed in 5 straight playoff appearances3 of those losses came against the Pacers.\n\n2,7 k upvotes : 274 commentaires\nr/nba · il y a 2 m.\nThis was an all time Great day of nba playoff basketball\n\n183 upvotes : 39 commentaires\nr/nba· il y a 2 a\nNBA team logos over time\n\n464 upvotes : 136 commentaires\nWhich NBA team did not have home court advantage until the NBA Finals?\n\n113upvotes:80 commentaires\nr/nba • il y a 2 m.\nNBA Teams That Never Met in the Playoffs (Same Conference)\n\n8 upvotes : 20 commentaires\nr/nba • il y a 2 m.\nWho would've won the 2018 NBA Finals if the Rockets beat the Warriors in game 7 of the WCF?\n\n34 commentaires\nr/algeria ·il ya 9j\nAnyknownAlgerianbasketballteams?\n\n4 upvotes : 16 commentaires\nr/pacers ·il ya 28j\nIf Pacers and Nuggies Go to Finals, Who Has Homecourt?\n\n4 upvotes : 16 commentaires\nr/canes · il y a 1 m.\nThe last time we won a double OT game in the first round of the playoffs\n\n58 upvotes- 6 commentaires\nr/AllAmericanTV.il y a1a\nWhat NFL team will Spencer play for?", "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nO Répondre\nMeece_\nAnd the argument that it prevents tanking falls somewhat short\nBefore the play ins, teams just gave up if they were like 5 or more games outside the 8 seed.\nNow damn near every teams fights for a play in spot or to keep themselves in the 6th seed or\nabove. It has revitalized the last third of the season.\nThen the play in games themselves are pretty fun too. Play ins have had nothing but positive\neffects for the NBA.\nThe chances of a 6-8th seed making the Finals is slim. Should we exlude them from the\nplayoffs entirely too? Feels silly to base things off their chances of making the Finals.\n\n\nO Répondre\njustmefishes\nThe play-in is worthwhile for its own sake. It's a few mini-Game 7s amongst not-great but not-\ncompletely-awful teams which makes for a nice appetizer going into the playoffs. Personally I\nfind it very interesting to see more flawed / average teams being put in that situation as you\nget to learn things about teams and players you otherwise wouldn't, because they'd either\nmiss the playoffs entirely or get bounced quickly in the first round by a much better team.\n\nre: the Mavs, I don't think they tanked, it was actually disastrous for them to miss the playoffs\nafter the Luka trade and it was almost entirely down to injuries. They got lucky in the lottery\nbut we know what their odds were, and it's really not worth tanking out of the play-in for such\nlow odds. A statistical fluke doesn't change that point.\n\n↑ 26 →O Répondre", '[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nO Repondre\nLadnil\nIt does prevent tanking. Just not 100% of it. But there are degrees of this\n\nO Répondre\nxelecunei\nI still think that the play-in is still a good idea. It just needs an overhaul.\nThey should just implement the play-in if the 7th and 8th seed is just 1-2 games ahead of the\n9th and 10th.\nIf the 7th seed is 4 or so games ahead, their spot should already be locked in. Same with the\n8th, if they are games ahead their spots should already be locked in.\nIt just doesn\'t make sense that an 8-game behind team having a shot at the play-offs.\n\nO Répondre\nelbosston\nIt\'s harder in basketball because usually the "better team" goes to the finals as basketball has less variance\nthan hockey due to how much harder it is to score in hockey\n\n\nsomeguy_3112\n2023 Heat Edit: just noticed that you asked for a team that had the home advantage in the finals. My bad', "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nO Repondre\nClownFundamentals · -11 j\nYeah, it'd really mess up their skates.\nO Repondre\nTeam_Ed·-11j\nNever in the NBA.\nThat's because Hockey is the favourite sport of the god of randomness and lower seeds win way more\noften than in basketball.\nThe NHL also has the same problem as the NBA of having the post-season be so much more intense that\nit's almost a different sport. What worked for a 110 point President's Trophy winner in the regular season\nmay not work at all in the playoffs.\nO Repondre\nareksoo ·-12j\nNever happened. For a team to make the final never having home court advantage you have to be the 5th\nseed. So the finals, needs a 6th or lower... but that's never happened because every finals contained at\nleast a 1st, 2nd or 3rd seed.\nO Repondre\nHeresTheAnswer\nyou could be any seed below 4th. If both teams were 8th seeds the one with better record would have\nhome court\nO Repondre\ndaymanahhhahhhhhh : -12 j\nThis has never happened in the nba.\nO Repondre\nSkinnecott · -12j\nif the lakers would have made the finals in 2023 it would have been heat vs lakers and only time heat had\nhomecourt would be finals. but denver beat them 3rd round and had homecourt over us\nO Repondre\nMaleficent_Resolve44 : -11 j\nHasn't happened yet. You'd need two proper low seeds to come out of both the west and east. Never\nbeen done before because the best teams usually get the highest seeds.\nO Repondre\nDr_Satan36·-12j\nsigto117·-12j", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\nvmpafq· -10j\nIf you filter for Reggie's prime years you would have to do the same for the others to make a fair comparison. Most of these guys have double the volume at least.\n\nO Repondre\nEyeFar9259·-10j\nReggie has had one of the greatest playoff scoring peaks. So this follows\n\nO Repondre\nHendo8888·-10j\nHow does rTS% work?\n\nO Repondre\nvmpafq · -10j\nrelative to league average TS%Ithink\n\nO Repondre\nRecommendationReal61:-10j\nPoints 1 and 2 can be true, but don't provide enough to support the argument proposed in point 3. There are at least a dozen other guards who unlike Reggie actually won MVPs and/or Finals MVPs, so maybe\nefficiency isn't the most important statistic in measuring a guard's value.\n\nName me one player who comes close to 14 playoff series wins with zero HOF teammates in their prime.\n-2\n\nOk so from 1991 to 2002 when Reggie averaged 24PPG on 17 shots a game, who exactly do you think was the number one option?\nHe's not a better player than any of the 2o I listed, ofc not bc there is more to the game than efficient scoring. But he definitely was a first option, and his resume is absolutely top 50 material. He won a lot for someone who never had a superstar teammate.\n\nHow many does Butler have?", "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nO Répondre\nsomeguy_3112\nYeah I missed that they asked for a team with home advantage in the finals, just edited my\ncomment\nDemonsReturns7 .-12j\nBut did they have home court adv in the finals though? I don't remember\nO Repondre\nhickok3 ·-12j\n Comm.du top 1%\nNo, Denver was the 1 seed iirc, and at the very least had home court.\nO Repondre\nrunevault · -11j\n Comm. du top 1%\nThe funny thing was the Nuggets took their foot off the gas after getting a 7 game lead over the 2\nseed Grizz and people worried they were throwing away home court in the finals because at least\nthe top 2 seeds in the east had better records.\nInstead Nuggets faced the Heat lol.\nO Répondre\nsomeguy_3112 · -12j\nYou're right, I missed the finals part in the post\nO Repondre\nYourWorstNightmare9·-12j\nThey would've had home court advantage in the Finals if the Lakers had beaten the Nuggets in the\nWCF that year.\nO Repondre\nwould really need a very lopsided difference between conference, like in 2008 when Golden State missed\nthe playoffs at 48-34 in the west but the Cavs could be a 5th seed at 45-37. That year, for example, had\nthe Suns and Rockets (both 55-27 and the 6th and 5th seed) made a run (not as crazy as it sounds, the\nLakers were 1st at only 57-25), with the Suns going to the finals, and the Magic (52-30) gotten hot and\nalso gone ot the finals, like they did next year, the Suns would have been the lower seed each round until\nthe finals\nO Repondre\nTearz_in_rain ·-11j", '[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nPlayoff riser\nThe modern NBA being the most efficient NBA isn\'t just about rule changes; it\'s that too, but moreso it\'s offensive strategy centered around maximizing efficiency, and iMO players who are collectively more talented than ever. No reason why the player with the highest absolute Ts% shouldn\'t be considered the most efficient in history\n\nO Répondre\nGrenScrin ·-10j\nDefinitionof"mostefficientfirstoption"+rTs%\n\nO Repondre\nSad_Bathroom1448·-10j\nAgreed. I get why rTs% exists, but you wouldn\'t say the fastest computer in 1955 is the fastest computer ever just because it\'s so much faster than the average computer in 1955.\n\nO Repondre\ncostelci·-10j\nYou could argue it had the best engineering though, as it was the furthest ahead of the competition operating with the same technology. different eras matters in any way is up to you I guess.\n\nO Repondre\nMalcolmSupleX·-10j\nReggieTS%?\n\nO Repondre\nNiviclades·-10j\nRelative True Shooting is my guess\n\nO Repondre\nKawhi Leonard\n112\nStephen Curry\n4147\nJerry West\n4457\nKareemAbdul-Jabbar\n5762\nKevin Durant\n4985\nCharles Barkley\n2833\nDirk Nowitzki\n3663\nLeBron James\n8289\nShaquille O\'Neal\n5250\nWilt Chamberlain\n3607\nNikola Jokic\n2580\nMichael Jordan\n5987\nJames Harden\n3895\nHakeem Olajuwon\n3755\nJulius Erving\n4580\nTim Duncan\n5172\nDwyane Wade\n3954\nGiannis Antetokounmpo\n2270\nKobe Bryant\n5640\nLarry Bird\n3897\n\nO Repondre\npick-and-hoop·-10j\nWow, Kawhi was basically one or two playoff runs from passing Larry Bird, that is so unexpected.', "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n↑ 26 →O Répondre\n\n\nMayBeAGayBee\nThe main benefit of the play-in is just the fact that it can keep most of the teams hovering\naround that 6-seed/7-seed boundary in a death race until the very end of the regular season\nin order to avoid the play-in.Plus 7 and 8 seeds are basically freebie first round series\nanyways. It's not as if 1 and 2 seeds losing in the first round has ever been particularly\ncommon even before the play-in.\n\n\nUmmm https://www.basketball-reference.com/teams/MIA/2023.html\nNot a 9/10, but a play-in team that made it to the finals.\n\n\nO Répondre\nalmondsandrice69\nit only exists for an extra 4 games of revenue, but i would not mind if they reverted it to the\nsystem from the bubble, where it only kicked in if the teams were within a certain number of\ngames of each other. in 2024, 8-seed Miami won 7 more games than the 9-seed Bulls &amp; this\nyear, the grizzlies won 8 more games than the 9-seed kings. there's absolutely no reason why\neither of those teams needed to have a play-in game.\n\nO Repondre\nLadnil\nIt does prevent tanking. Just not 100% of it. But there are degrees of this", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\npick-and-hoop·-10j\nWow, Kawhi was basically one or two playoff runs from passing Larry Bird, that is so unexpected.\n\nO Repondre\ntheeExample· -10j\nWas? You know he's still playing right? Lol\n\nO Repondre\ncomposer_7 . -10j\nNice to see Charles Barkley here too. Most people think he was just rebounds like Dennis Rodman and not a great scorer too.\n\nO Repondre\nSerious-Question281 · -10j\nHe did score 8 points in 9 seconds once. Very efficient\n\nO Repondre\nTarrot469·-10j\nOne thing that stands out is how high Jerry West is without the 3-point line to help boost TS. And he's the best guard defender of his era. People massively sleep on him and he should be right on the top 10 border.\n\nO Repondre\nTorkzilla·-10j\nReggie was my favorite player growing up and I definitely think he can hang with just about any shooting\n\nO Repondre\nSterlingStRose·-10j\nMight be why he's in the hall of fame\n\nO Repondre\nben10toesdown ·-10j\nDWade is definitely ahead of Reggie.\n\nO Repondre\nGreedyWarlord · -10j\n3rd best SG of all time, arguably, top 5 definitely. Won 3 chips. One with a waning Shaq. That doesn't mean he was necessarily a more efficient scorer. there is an argument to say that Reggie may be the 5th most valuable guard for a single franchise ever after Jordan, Magic, Curry, and Kobe I'm just arguing this point. And after rereading it, Zeke is ahead of Reggie too\n\nO Repondre\ndjinngerale : -10j\ntop 5 definitely\nJordan, Kobe, Wade, Iverson and who else in your books?"]</t>
+          <t>["[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n183 upvotes : 39 commentaires\nr/nba· il y a 2 a\nNBA team logos over time\n\n464 upvotes : 136 commentaires\nr/nba/comments/11066qq/which_nba_team_did_not_have_home_court_advantage/\n\n113upvotes:80 commentaires\nr/nba • il y a 2 m.\nNBA Teams That Never Met in the Playoffs (Same Conference)\n\n8 upvotes : 20 commentaires\nr/nba • il y a 2 m.\nWho would've won the 2018 NBA Finals if the Rockets beat the Warriors in game 7 of the WCF?\n\n34 commentaires\nr/algeria ·il ya 9j\nAnyknownAlgerianbasketballteams?\n\n4 upvotes : 16 commentaires\nr/pacers ·il ya 28j\nIf Pacers and Nuggies Go to Finals, Who Has Homecourt?\n\n4 upvotes : 16 commentaires\nr/canes · il y a 1 m.\nThe last time we won a double OT game in the first round of the playoffs\n\n58 upvotes- 6 commentaires\nr/AllAmericanTV.il y a1a\nWhat NFL team will Spencer play for?\n\n8 upvotes : 19 commentaires\nr/nba · il y a 13 a\nNBA Court Explained", "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n4 upvotes : 16 commentaires\nr/canes · il y a 1 m.\nThe last time we won a double OT game in the first round of the playoffs\n\n58 upvotes- 6 commentaires\nr/AllAmericanTV.il y a1a\nWhat NFL team will Spencer play for?\n\n8 upvotes : 19 commentaires\nr/nba · il y a 13 a\nNBA Court Explained\n\n25 upvotes : 19 commentaires\nr/nba· il ya6a\nCan someone explain to me what it means for a team in the playoffs to take home court?\n\n1upvote:14commentaires\nr/nba · il y a 3 m.\n\n16upvotes:9commentaires\nr/lakers • il y a 2 m.\n[Buha] Luka Doncic notes that this is the first time he'll have home-court advantage in a playoff series.\n\n1,5kupvotes·53commentaires\nBest NBATeams That Never Wona Championship\nBestNBARecord82-GameSeason", '[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n101 upvotes : 44 commentaires\nr/nba·il y a 11j\n[Smith] This is now reality. Thunder vs Pacers will be the first NBA Finals since the luxury tax has been in effect where neither team was a taxpayer for that season.\n\n11 k upvotes : 948 commentaires\nr/hockey · il y a 13j\nThe Oilers are the first Canadian team to have home-ice advantage in the Stanley Cup Finals since the 2011 Vancouver Canucks\n\n2,5 k upvotes : 226 commentaires\nr/nba·ilya 11j\nThe Knicks have now lost to a lower seed in 5 straight playoff appearances3 of those losses came against the Pacers.\n\n2,7 k upvotes : 274 commentaires\nr/nba · il y a 2 m.\nThis was an all time Great day of nba playoff basketball\n\n183 upvotes : 39 commentaires\nr/nba· il y a 2 a\nNBA team logos over time\n\n464 upvotes : 136 commentaires\nr/nba/comments/11066qq/which_nba_team_did_not_have_home_court_advantage/\n\n113upvotes:80 commentaires\nr/nba • il y a 2 m.\nNBA Teams That Never Met in the Playoffs (Same Conference)', "[Contexte: How is it that the two best teams in the playoffs based on stats, having a chance of playing against each other in the Finals, is considered to be a snoozefest?]\nExpiredDeodorant·-15j\nI can watch 100 OKC defensive possessions and in 100 of them there will be something that\nshould be called for a foul\n 1  O Repondre\n\nReggie Miller is the most efficient first option in NBA playoff history\n1,3kupvotes·317commentaires\n\nThe Finals is one of the GOATs when you consistently play with a team.\n\nFor the fourth straight year, the loser of the ECF went on to go to the finals the very next year.\n\n[Highlights] All the 78 fouls by Karl-Anthony Towns in the 2025 NBA Playoffs.\n\nTeams are now 54-20 (.730) this postseason when having fewer turnovers than their opponents.\nIt's the best winning percentage in a single postseason in NBA history (minimum 20 total games).\n\nThunder vs. Pacers: A look at the stats for both teams in the playoffs so far", '[Contexte: How is it that the two best teams in the playoffs based on stats, having a chance of playing against each other in the Finals, is considered to be a snoozefest?]\nO Repondre\n\nhoppergym ·-15j\nWho considers it to be a snooze fest? Please cite Sources\n\nO Repondre\n\ncody_d_baker ·-15j\nAgreed, I\'m tired of this narrative on r/nba, all I\'m seeing is constant excitement over the small market\nteams and people saying the ratings don\'t matter\nO Repondre\n\nDelusional_Donut ·-15j\nIthink it\'s carry-overdiscoursefromlastyear\'s playoffs,casual social media sports content creators\nwho don\'t actually watch the sport just saying whatever so they can post 3 YouTube shorts a day\nO Repondre\n\nhoppergym ·-14j\nWho? What nba media? That\'s all I\'m asking.\nO Repondre\n\nTerrible_Shelter_345·-15j\nIt\'s probably just salty Celtics fans, Knicks fans, Jokic stans, and Ant stans all bitching online\nNo one in real life would ever be talking "tv ratings" at the bar or the kickback watching a ball game\nImao\n个 2\nRepondre']</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>D'après les données disponibles dans le contexte fourni, je ne peux pas comparer les statistiques de rebonds des équipes à domicile et à l'extérieur. Les extraits de Reddit et les discussions ne contiennent aucune information sur les performances en rebonds selon le lieu des matchs (domicile/extérieur).
-Si tu veux une analyse précise, je te conseille de consulter des sources spécialisées comme **Basketball-Reference**, **NBA Advanced Stats** ou **ESPN Stats**. Veux-tu que je t’aide à trouver ces données ailleurs ?</t>
+          <t>Désolé, les infos ne sont pas disponibles dans la base de connaissances de ce RAG.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Information non disponible : les données ne distinguent pas les matchs joués à domicile de ceux joués à l'extérieur.</t>
+          <t>Désolé, les infos ne sont pas disponibles dans la base de connaissances de ce RAG.</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -759,7 +752,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0.7167769097543741</v>
+        <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -775,97 +768,85 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Quelles équipes ont le plus impressionné lors des playoffs ?</t>
+          <t>Quelle meteo pour demain à Nantes?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>["[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\ninshamblesx · -1 m.\nwolves by a mile\n\nTemperedTorture · -1 m.\nWolves by far. Particularly Edwards. I hadn't seen any Wolves games going into the playoffs, so I had no\nclue just how amazing Edwards was and he's really in the middle of a massive leap these playoffs. They\nhave a strong team -- and that's important these playoffs more than ever. Hero/iso ball is essentially dead\nbecause of how good defences have gotten.\nIt's been a joy to watch the Lakers/Wolves series and I'm becoming a huge fan of Ant. OKC, Celts and Cavs\nare performing up to expectation. Kinda always knew that Gsw would muscle through because of their\nsheer playoff and championship experience. Wasn't expecting the way Wolves have torn into the Lakers\nand exposed their lack of roster depth.\n\nOther-Owl4441\nLakers team is pretty flawed and they're exploiting them well. With Wolves the question is still if\nthey're a tier below. Obviously OkC is a tough matchup for anyone but I don't think Wolves have\nproved anything they didn't show last year.\n\nBrofessor-\nTimberwolves have beat OKC 2 times this season btw\n\nNiceguydan8 · -1 m.\nFor me it's less the teams and more so players.\nPaolo is the big standout for me\n\nProof-Umpire-7718\nAuteur-rice top 1%\nMagic need to get some competent offensive playsrs, particularly some shooters, around him and\nFranz this offseason.", '[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\n2. Jaden has taken an incremental step on offense, becoming much more willing/able to dribble-drive into short range pull-ups and attempts at the rim. Again, he would do this last season but now he\'s doing it with greater consistency.\n\n3. Donte as a bench creator/ball-handler who can hold his own somewhat on defense is a huge addition that helps mitigate Conley having down streaks.\n\n4. Julius is less a dynamic scorer compared to KAT but he still flls the role as a "get-a-bucket" iso guy. He\'s also a better passer off the dribble although that hasn\'t been as apparent in this series so far.\n\nYeah I know Donte hasn\'t played well this series but I thought a guy like that to come off the bench and at least take some pressure off is definitely something they were missing last year\n\nI definitely thought the Wolves trading Kat was a huge downgrade but they definitely have adjusted to the new roster and look as good as ever.\n\nIndiana but I kind of expected it. I really think they have a legit shot against the Cavs next round. Their offense is no joke.\nWho are teams in the playoffs that have impressed you ? : r/nba\n\nSe connecter\n\nWho are teams in the playoffs that have impressed you ? : r/nba\n\nAnyone else feel like these playoffs are the most unpredictable in years?\n\nI think we should cherish the parity in the nba, because it\'s not going to last.', '[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nKingmav24 · -1 m.\nthis might be the least watched finals of all time\n\nDeep down they all still want a Celtics-Lakers final\n\ndelta_velorum : -1 m.\nIf it\'s a Wolves-Pacers final, I\'m switching to watching the WNBA\n\nsmkmn13.-1 m.\nRandle shooting 45% from three is a massive boost for a 33% career guy. Balancing out\nDonte/NAW/Copley\'s rough shooting.\n\nRandomerThanYours·-1m.\nMagic have been solid but I wouldn\'t really call it taking us to the brink. Atlanta a couple years ago was\nthe real scary first round.\n\nBoneslIX · -1 m.\nMagic is one of those "if they figure it out, they\'re gonna be scary" examples. I\'ve been pretty high on\nthem for 2+ seasons. Hoping for health for them next year. They will be a regular conference\ncontender if they get a little more 3pt shooting and continue to ride the growth of Paolo and the\nWagners.\n\n[supprimé] · -1 m.\nBut with the magic you\'re always moments away from a serious injury\n\nSteamingHotChocolate·-1 m.\nthis series is certainly taking me to the brink of insanity for that reason yeah\n\nEasy_Magician_925 ·-1 m.\nhl Magic have been down 2 of their more impactful players all series and could easily be tied 2-2 let\nalone up 3-1.\n\nhollow-ataraxia·-1m.\nTrae won\'t get credit for it because he went cold in the second half of game 6 and he started the\nseries slow but that game 5 and first half of game 6 was some of the best basketball I\'ve ever seen\nhim play. He single handedly almost willed us to a game 7 but ran out of gas.', "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nTallnFrosty · -1 m.\nuntil franz fixes his shooting, i don't think 'dynamic' is the right word for him\n\nlegendofthededbug · -1 m.\nthepeachgod . -1 m.\nIndiana is gonna have a better chance at beating Cleveland than people will give them\n\nSiakam is themost underrated playerin the league as far as impact towards winning.if that team's\nclicking, which they seem to be with Hali dishing the way he is right now, they're a tough out for\nanyone\n\nshhhhhhhwish · -1 m.\nBy far the toughest series last year for the Celtics. I think we'll get a Celtics Indy rematch tbh... no one\nwill see it coming but it wasn't a fluke Indy got there last year\n\nYankeeknickfan · -1 m.\nIt's impressive that they're finally not just scraping by a team that's injured and straight up\nDominating a worse team. Definitely better than last year\nBut the bucks are awful. Really don't get why dominating them says anything about Cleveland\n\nPistons are one shot creator from being an ECF contending team imo.\n\nMannerSuperb Ao\nbefore his injury\n\naenima1991 : -1 m.\n10000% I keep thinking that - where would they be w Ivey. Probably up in this series.\n\nOther-Owl4441 : -1 m.\nLove Ivey but isn't the ideal profile for that missing piece a shot creator who's a knockdown\nshooter, instead?\n\nPootieTooGood\nI'm praying that they do not believe Ty Jerome is their answer since they're the team with the cap\nspace to pry him away from us\n\ninshamblesx · -1 m.\nwolves by a mile", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nxWolfsbane : -1 m.\nMagic have no shooters. It's like watching the early 2000s. I don't mind it, but they won't win\nwithout a 3 ball.\n\nARGHETH · -1 m.\n\njustletmeregisteryou · -1 m.\n+Auteur-ricetop1%\nI'm sorry, but you're impressed with... The Magic?\nAnyway, I hate it but I gotta give credit to Indiana. They impressed me last year too ad honestly, that\noffense is capable of beating literally everyone lol. not saying they're gonna win it all or anything, but\nCarlisle and the players deserve massive credit\n\n←\n\nKlumber · -1 m.\nRespect. I will always wonder 'what if' about last year's run without Giannis, but this year I think the\ndifference is there.\n\nMannerSuperb AO . -1 m.\nPaolo and Franz have been a dynamic wing duo this whole series agaisnt one of the best defensive\nteams in basketball plus the defending champs. Yes the supporting cast has been laughably bad at\ntimes around them offensively but they guard their asses off and really giving the Celtics a fight\ndespite missing Suggs and the other Wagner brother. I thkkk their floor spacers and average PG away\nfrom being an true contender\n\ngeorgiosauce : -1 m.\nMagic are down 3-1 despite injuring 3 Celtics starters along the way, they're solid trash\n\nPeachTreeDish91 · -1 m.\nYou really seem like the type of dude who spends 10 minutes watching the youtube highlights\nwhile checking the box score, then spends the next 60 minutes typing bs out the ass on reddit", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nNo_Albatross916 . -1 m.\nIndiana and Minnesota to me\n\n57\n\nthereticent · -1 m.\nPistons for me. Not surprised, just impressed with them\n\nProof-Umpire-7718 · -1 m.\nWolves\n\n61\nWolves are not surprising if you had watched them, I had picked them to beat the Lakers in six and\nwas specifically the team I wanted to dodge in the first round the most.\nThe have the highest ceiling of all the teams outside of Okc because they can be both elite offensively\nand defensively. Their only real flaw is decision making at times, but even then Ant has improved\nhugely on that end.\nI think they were ultimately under estimated as too many crowned the Lakers as being better than\nthey are actually are. Especially after the OKC H2Hs where their shooting output just wasn't very\nrealistic of who they were in a Playoff setting.\nI think the next best team is the Clippers, but man they have definitely found ways to lose games\nagainst the Nuggets.\nBut ultimately think it's going to end up pretty comfortably a OKC-MiN WCF and that is going to be\nan insane series.\n\nMaybe to you but we got humbled last year\n\nCade. Dude needs to seriously cut down on the turnovers, but he's a bucket.\n\nI get frustrated with his sloppy turnovers a lot but he's kind of in the position he has to. Too many possessions where\nwe can't even get the ball inside 30 feet of the basket if he doesn't touch the ball", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nthat it has not panned out with him\nYes, Iwould be excited to see whatkind of numbers Paolo could put up if hehad more creation and shooting.\nHell, I would be excited to see what Paolo's numbers look like if the Magic were just ONE of the slowest pace team and just ONE of the lowest scoring teams and not dead last in both.\nI wonder what he would average if the Magic were 25th in pace and 25th in scoring versus 30th.\n\nPaolo and Cade both are mature difference makers. They look like they can carry on their shoulders.\n\npistons for sure. despite the crying about the whistle being too loose or too tight depending on the outcome, despite the knicks being incredibly healthy and the pistons being down ivey and now stew, they have been in every single game and cade is proving why he was the correct #1 pick in a draft that includes mobley, barnes, wagner, and sengun. once they are able to replace tobias (great signing for a stopgap veteran) through either trade, FA, or draft, they will be a top 5 team in the east for many years.\n\nI would say the Twolves.I hadn't watched them much this season but their offense just looks so much better than last year. Ant seems to trust his teammates a lot more (obviously helps when they are making shots) and they aren't completely reliant on him playing iso in the end of games\n\nmajority of his attempts from dribble pull-ups. He was good in this area before but now he's elite and it's obviously a vital component to closing out games and stifling runs.", "Who are teams in the playoffs that have impressed you ? : r/nba\n\nMannerSuperb\nWho are teams in the playoffs that have impressed you ?\nFor me it's the magic. Despite awful shooting , they have really taken the defending champs to the brink. I'm a\nlittle biased as a Duke fan but Paolo and Franz are absolute dogs and my favorite young wing duo in the\nleague those guys have shown they are built for playoff basketball with their shot making ability and\ncompeting defensively. I truly hope orl can get those kids some real shooters and a true point guard theirs\nanother level their games and overall team can reach if they simply had some floor spacing and average guard\nplay around them.\n\n31\n236\n\nNotWD . -1 m.\nAnt's been a machine as expected, but Randle's genuinely beating the beyblade allegations and it's so\nnice to see\n\n186\n\nMG_MN .-1 m.\nRandle has been a revelation. His bully ball has worked perfectly on offense, and his physically is a big\nreason LeBron has run out of gas\n\n55\n\nGbaby245 : -1 m.\nRandle knows he can out muscle most guys one on one, and then makes the correct read when\ndoubles come. He also plays defense with his chest, not hands so he doesn't get the fouls Kat did.\nLuka and Bron can't just shove Randle out of the way on every drive.\n\n32", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\n32\n\nYou knew when I KNEW it would work? When Rashad McCants co-signed it.\nThe biggest revelation to me has been Randle's commitment on the defensive end. He looks\nmuch more engaged and focused right now. I'm hoping he won't stay as interested in the\nsecond round (if he beats his former team and if the Warriors beat the Rockets).\n\nflyingcrayons · -1 m.\nRandle has been past beyblade mode for years now, unfortunately he's been hurt the last few times\nthe Knicks were in the playoffs and everyone was watching so people still think he's the Randle from\n4-5 years ago\n\n36\n\nTappedRidgeline : -1 m.\nRandle's playoff reputation really ignores the circumstances. He had 1 actual poor playoff series\nagainst the Hawks, with 3 million year old DRose as the next best player on the roster, and then\nhad like 3 ankle sprains in 2 weeks the next time the Knicks made the playoffs. This is really his\nfirst opportunity to shine, and it's been fun to watch him and donte in these playoffs on another team.\n\nbronet · -1 m.\nHoping we get T-wolves vs Pacers in the finals so we get some real beyblade duel action\n\n31\n\naenima1991 : -1 m.\nWhat's the beyblade joke I don't get it\n\nbronet ·-1 m.\nBoth Randle and Siakam used to spam spin moves every time they went to the basket\n\naenima1991 : -1 m.\nAhh haha\n\nKingmav24 · -1 m.\nthis might be the least watched finals of all time\n\nDeep down they all still want a Celtics-Lakers final", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nCade has really impressed with his play but even more so with his leadership. I think Detroid has a\nmaturity and emotion problem which can be buffed out with age and experience. He's holding both\nhimself and his teammates accountable. Him pushing his rookie away yesterday to keep him in check,\nchill him out and stop him from getting a stupid tech was some real shit.\n\nIt's a talent issue. Stew and Holland definitely run hot but that's not the issue. The team feeds off that a lot of times. They just don't have a secondary scoring\noption outside of Cade especially with Ivey hurt. A lot of this is being passed on to Dennis\nSchroeder/Malik Beasley/Tobias Harris which is a good patch job for this season but it's not\nreliable or what you want in a playoff series.\n\nHe also needs to seriously work on his jumper. His 3-ball isn't very good. That needs to be\nnorth of 35% to explode.\n\nWas north of 35% this season.\n\nthey don't really have a secondary playmaker. Their second best shot creator\nShroeder. He's being asked to do a lot as the sole focus of the opposing team.\n\nYou must hate good offense, I have been disgusted watching the Magic play\n\nGood offense is a lot harder to come by in playoff basketball tho. Games are more physical and lower\nscoring. Warriors have a great offense and struggling against a physical rockets defense\n\nTheMagicoffenseisbasketballterrorism."]</t>
+          <t>["[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n183 upvotes : 39 commentaires\nr/nba· il y a 2 a\nNBA team logos over time\n\n464 upvotes : 136 commentaires\nr/nba/comments/11066qq/which_nba_team_did_not_have_home_court_advantage/\n\n113upvotes:80 commentaires\nr/nba • il y a 2 m.\nNBA Teams That Never Met in the Playoffs (Same Conference)\n\n8 upvotes : 20 commentaires\nr/nba • il y a 2 m.\nWho would've won the 2018 NBA Finals if the Rockets beat the Warriors in game 7 of the WCF?\n\n34 commentaires\nr/algeria ·il ya 9j\nAnyknownAlgerianbasketballteams?\n\n4 upvotes : 16 commentaires\nr/pacers ·il ya 28j\nIf Pacers and Nuggies Go to Finals, Who Has Homecourt?\n\n4 upvotes : 16 commentaires\nr/canes · il y a 1 m.\nThe last time we won a double OT game in the first round of the playoffs\n\n58 upvotes- 6 commentaires\nr/AllAmericanTV.il y a1a\nWhat NFL team will Spencer play for?\n\n8 upvotes : 19 commentaires\nr/nba · il y a 13 a\nNBA Court Explained", '[Contexte: How is it that the two best teams in the playoffs based on stats, having a chance of playing against each other in the Finals, is considered to be a snoozefest?]\nTerrible_Shelter_345·-15j\nIt\'s probably just salty Celtics fans, Knicks fans, Jokic stans, and Ant stans all bitching online\nNo one in real life would ever be talking "tv ratings" at the bar or the kickback watching a ball game\nImao\n个 2\nRepondre\n\nND7020·-15j\nthat\'s true or not anyway); and\n2. Those saying the Thunder will win easily. I think (and hope) that\'s wrong. If you believe the Thunder\'s\ndefense will just smother the Pacers, then yes, it will be a snooze, particularly as they don\'t play an\nexiting brand of basketball.\nBUT the Pacers play very exciting ball, Carlisle is a hell of a coach, their PG doesn\'t turn the ball over, and\nthey are great at dictating the pace of games. They\'ve been counted out a lot. I\'m not counting them out\nin the finals.\n+9+\nORepondre', '[Contexte: How is it that the two best teams in the playoffs based on stats, having a chance of playing against each other in the Finals, is considered to be a snoozefest?]\nO Repondre\n\nhoppergym ·-15j\nWho considers it to be a snooze fest? Please cite Sources\n\nO Repondre\n\ncody_d_baker ·-15j\nAgreed, I\'m tired of this narrative on r/nba, all I\'m seeing is constant excitement over the small market\nteams and people saying the ratings don\'t matter\nO Repondre\n\nDelusional_Donut ·-15j\nIthink it\'s carry-overdiscoursefromlastyear\'s playoffs,casual social media sports content creators\nwho don\'t actually watch the sport just saying whatever so they can post 3 YouTube shorts a day\nO Repondre\n\nhoppergym ·-14j\nWho? What nba media? That\'s all I\'m asking.\nO Repondre\n\nTerrible_Shelter_345·-15j\nIt\'s probably just salty Celtics fans, Knicks fans, Jokic stans, and Ant stans all bitching online\nNo one in real life would ever be talking "tv ratings" at the bar or the kickback watching a ball game\nImao\n个 2\nRepondre', "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n4 upvotes : 16 commentaires\nr/canes · il y a 1 m.\nThe last time we won a double OT game in the first round of the playoffs\n\n58 upvotes- 6 commentaires\nr/AllAmericanTV.il y a1a\nWhat NFL team will Spencer play for?\n\n8 upvotes : 19 commentaires\nr/nba · il y a 13 a\nNBA Court Explained\n\n25 upvotes : 19 commentaires\nr/nba· il ya6a\nCan someone explain to me what it means for a team in the playoffs to take home court?\n\n1upvote:14commentaires\nr/nba · il y a 3 m.\n\n16upvotes:9commentaires\nr/lakers • il y a 2 m.\n[Buha] Luka Doncic notes that this is the first time he'll have home-court advantage in a playoff series.\n\n1,5kupvotes·53commentaires\nBest NBATeams That Never Wona Championship\nBestNBARecord82-GameSeason", '[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n101 upvotes : 44 commentaires\nr/nba·il y a 11j\n[Smith] This is now reality. Thunder vs Pacers will be the first NBA Finals since the luxury tax has been in effect where neither team was a taxpayer for that season.\n\n11 k upvotes : 948 commentaires\nr/hockey · il y a 13j\nThe Oilers are the first Canadian team to have home-ice advantage in the Stanley Cup Finals since the 2011 Vancouver Canucks\n\n2,5 k upvotes : 226 commentaires\nr/nba·ilya 11j\nThe Knicks have now lost to a lower seed in 5 straight playoff appearances3 of those losses came against the Pacers.\n\n2,7 k upvotes : 274 commentaires\nr/nba · il y a 2 m.\nThis was an all time Great day of nba playoff basketball\n\n183 upvotes : 39 commentaires\nr/nba· il y a 2 a\nNBA team logos over time\n\n464 upvotes : 136 commentaires\nr/nba/comments/11066qq/which_nba_team_did_not_have_home_court_advantage/\n\n113upvotes:80 commentaires\nr/nba • il y a 2 m.\nNBA Teams That Never Met in the Playoffs (Same Conference)']</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>D’après les discussions des fans sur Reddit, **les Timberwolves du Minnesota** sont clairement l’équipe qui a le plus impressionné lors de ces playoffs, selon plusieurs commentaires récurrents. Voici les points clés qui ressortent :
-- **Ant Edwards** est salué comme une révélation, avec une progression majeure en playoffs (dribble-drive, iso clutch, leadership). Les fans soulignent son adaptation à un rôle plus complet, loin de l’iso-ball pur.
-- **Collectif solide** : Malgré des doutes sur leur profondeur de banc, les Wolves ont dominé les Lakers (notamment en exploitant leurs faiblesses défensives) et prouvé qu’ils pouvaient rivaliser avec les meilleures équipes.
-- **Potentiel défensif/offensif** : Certains fans les voient comme une équipe capable d’être *elite* des deux côtés du terrain, avec une marge de progression (décisions parfois risquées, mais aussi une cohésion en hausse).
-**Autres équipes citées** (mais moins consensuelles) :
-- **Indiana Pacers** : Leur attaque est jugée "capable de battre n’importe qui" (même si leur parcours reste surprenant). Leur matchup contre Cleveland est attendu avec intérêt.
-- **Orlando Magic** : Malgré un manque criant de shooters, Paolo Banchero et Franz Wagner ont tenu tête aux Celtics (malgré des blessures), avec une défense agressive. Leur potentiel futur est souligné (si ils ajoutent des tireurs).
-- **New York Knicks** : Julius Randle est en pleine renaissance (défense engagée, bully ball efficace), effaçant son image de "beyblade" des années passées.
-- **Detroit Pistons** : Cade Cunningham impressionne par son leadership et sa maturité, malgré un roster limité. Leur progression est perçue comme un signe positif pour les années à venir.
-**À noter** : Les Warriors (expérience) et le Thunder (OKC) sont aussi mentionnés, mais plutôt comme des équipes *attendues* que *surprenantes*.
----
-*En résumé* : **Les Wolves trustent la palme**, suivis de près par Indiana et Orlando pour leur parcours inattendu. Les débats tournent surtout autour de leur capacité à tenir la distance face aux favoris.</t>
+          <t>Désolé, je ne peux répondre qu'à des questions concernant la NBA.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>D'apres les commentaires, les plus impressionnants sont les Wolwes (Minnesota) et les Indiana Pacers</t>
+          <t>Désolé, je ne peux répondre qu'à des questions concernant la NBA.</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8516508608821279</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9861111110987848</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.4303550713287926</v>
+        <v>1</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>simple</t>
+          <t>hors_scope</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>rag_fallback_after_sql_fail</t>
+          <t>rag_no_tool_call</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Combien de fois Reggie Miller a été all-star?</t>
+          <t>Selon l'auteur du post 'Who are teams in the playoffs that have impressed you?', quel duo de jeunes ailiers du Magic cite-t-il comme son duo préféré de la ligue ?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>["[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nIn game 7 against the Bulls in 98 it took Jordan pretty much going all out to make sure Miller never got a good look on any of his shots in that 4th quarter just to shut him down. So, it wasn't the easiest strategy and it took 2/3 GOAT-level players in Shaq, Kobe and MJ to make Miller ringless.\nBut, yeah, the ball-handling/ball-in-hand and creation part of the game is where someone with higher volume is likely more dangerous than Miller: a player that is more skewed towards being a pure shooter.\nAll of that being said, it's very possible that Miller is just one of the best versions of a player that would've gone down as an All-time #2 or 1B Option. It's easily possible he would've won more had he been paired with a player/team that had a better #1/1A option.\nA good example: put Miller on that mid-2000s Detroit team instead of Rip Hamilton. I'd say that's mostly an upgrade in every way: Miller is a better 3pt shooter than Rip and probably matches or exceeds him in everything else. Miller probably even wins finals MvP instead of Billups.\nI think, to some degree, Reggie was just overtasked on the offensive end and all the crazy feats he pulled off against teams in the East was because he was able to exceed his expectations as a player with that more limited skill-set.", '[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nPrestigious-Ad9921·-10j\nTim Hardaway is?\nOof.\nI\'ve started calling it the "Hall of Really Good."\nThat fits better.\n\nthesch ·-10j\nComm. du top 1%\nGood thread for the people who call Reggie overrated because they took one look at his bbref page and saw that he only made 3 all-NBA teams. Us uncs who were around then know he was the real deal.\nYep. Maybe the simplest argument in favor of Reggie Miller - he was the best player on a perennial playoff team for over a decade. Just a winning basketball player.\n\nBest player on a team that made the Finals, best player on one of the two squads team that took the 90\'s Bulls Championship teams to seven games.\n\nHis peers respect him so much that Reggie himself gets overwhelmed. I remember in the show Open Court when they discussed the next 25 best players and all of them said Reggie but Reggie insisted to not put him there.\nHis peers knew how hard it is to carry a franchise, a relatively small franchise, to the championship.\n\nYup, real ones know.', '[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\n\navd318.-7j\nReally illuminates how useless efficiency is as a metric\n\nO Repondre\n\nimperialmoose · -10j\nInteresting little set of stats! Regarding that last sentence, you\'re not accounting for all sorts of parts of\nthe game. It would be foolish to base his ranking all time purely off one stat. But you could argue he\'s\ncrazy, he made all NBA 3 times. Part of that may have been playing in Indiana, but partly he also wasn\'t\nthat good. Of the NBA 75, he\'s definitely in the bottom 20.\n\n\nHe was that good in the playoffs. He was Jamal Murray on steroids in the he greatly increased his\noutput once the games mattered. You can\'t just look at his regular season accolades and use that as\nan argument. He was plain and simple an absolute monster in the playoffs.\n\n\nI remember, I was there. I don\'t have any issue with OP saying Miller was a great playoff riser - we\nknow! I was addressing the final statement OP made; that he was the 5th most valuable franchise\nguard ever. He simply wasn\'t. There was one season I tried to argue with my buddies that he was a\ntop 10 player in the league. Even that was seen as a stretch. Like, he was never in an MVP\ndiscussion or even close.\n\nIf the argument is "he stayed with Indiana for a really long time, so he overall was more valuable\nto Indiana than Wade was to Miami"...I guess? Maybe?', "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\ndjinngerale : -10j\ntop 5 definitely\nJordan, Kobe, Wade, Iverson and who else in your books?\n\nO Repondre\nGreedyWarlord · -10j\nIt is pretty hard for me to choose the 5th one. Harden would be my choice, since I consider West a PG. Followed by Drexler and Gervin.\n\nO Repondre\nWhatever801 : -10j\nYeah Reggie is one of those guys where you have to really watch him to understand what he was like. Stats usually don't do it justice (well I guess this one does). Took the 98 bulls to 7.\n\nO Repondre\nJohnBlunt·-10j\nIt's funny because Reggie is probably the consensus worst player on this list\n\nO Repondre\nChrisclc13·-10j\nI think the most surprising take to me is that Larry Bird is at the bottom of this list.\n\nO Repondre\nwolfpack_57·-10j\nI wasn't around to watch, but wasn't he pretty reliant on screens to get open, and took less shots because he couldn't self-create? I think that takes away from the first option assertion because self creation should IMO be a part of first option status.\n\nO Repondre\ndevvinitely · -10j\nThis is why Ijoined this subreddit. I love this stuff\n\nO Repondre\nAcEr3_·-10j\nYeah Reggie is extremely underrated. Of course he's part of the top 75 but people do not truly understand fully how great Reggie was. I feel like over time more and more people are becoming aware which is good.", '[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nElyx_117 · -10j\nI like your 3rd point. Arguable but I like it. His longevity and consistency is often overlooked.\n\nfitzvery·-10j·Modifié il y a-10j\nIdk Reggie was great for a long time but saying he\'s more valuable then Jerry West, Oscar Robertson, or DwyaneWade is wild\n\nUniversityOk5928 · -10j\nAlso great for a long time for one franchise.\n\nOptism2·-10j\nWade still beats him easily cmon now\n\nUniversityOk5928 · -10j\nThe question was who is the most valuable to a franchise.\nYall love arguing without reading the question\n\nmacandcheeser · -10j\nI don\'t think Reggie vs Wade is a wild comparison. I\'d agree Wade had the higher peak, but Reggie was a stud for a long time, and always available.\nReggie is way ahead of Wade in career win shares. Reggie also slightly ahead in WS/48, and VORP.\nWade ahead in BPM\n\nGoblinTradingGuide·-10j·Modifié il y a-10j\nWhat OP has illustrated is basically the reason why Reggie is in the Hall of Fame. I know his selection was controversial but Reggie was a certified bucket getter.\n\nEntertainmentAOK ·-10j\nI mean if Tim Hardaway is in the HOF, Reggie definitely deserves to be there.\n\nPrestigious-Ad9921·-10j\nTim Hardaway is?\nOof.\nI\'ve started calling it the "Hall of Really Good."\nThat fits better.', "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\npick-and-hoop·-10j\nWow, Kawhi was basically one or two playoff runs from passing Larry Bird, that is so unexpected.\n\nO Repondre\ntheeExample· -10j\nWas? You know he's still playing right? Lol\n\nO Repondre\ncomposer_7 . -10j\nNice to see Charles Barkley here too. Most people think he was just rebounds like Dennis Rodman and not a great scorer too.\n\nO Repondre\nSerious-Question281 · -10j\nHe did score 8 points in 9 seconds once. Very efficient\n\nO Repondre\nTarrot469·-10j\nOne thing that stands out is how high Jerry West is without the 3-point line to help boost TS. And he's the best guard defender of his era. People massively sleep on him and he should be right on the top 10 border.\n\nO Repondre\nTorkzilla·-10j\nReggie was my favorite player growing up and I definitely think he can hang with just about any shooting\n\nO Repondre\nSterlingStRose·-10j\nMight be why he's in the hall of fame\n\nO Repondre\nben10toesdown ·-10j\nDWade is definitely ahead of Reggie.\n\nO Repondre\nGreedyWarlord · -10j\n3rd best SG of all time, arguably, top 5 definitely. Won 3 chips. One with a waning Shaq. That doesn't mean he was necessarily a more efficient scorer. there is an argument to say that Reggie may be the 5th most valuable guard for a single franchise ever after Jordan, Magic, Curry, and Kobe I'm just arguing this point. And after rereading it, Zeke is ahead of Reggie too\n\nO Repondre\ndjinngerale : -10j\ntop 5 definitely\nJordan, Kobe, Wade, Iverson and who else in your books?", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nFuck if dame is in then reggie should be there no question.\n\nI can believe that. Saw his whole career as a Knick fan and he didn't shoot as much by today's standards but I barely remember a time the guy missed\n\nHolly shit Jerry\n\nTim Hardaway was his teammate and in the HOF.\n\nkeep in mind that he didn't take nearly as many FGA per game as stars did back then or now. Like, he'd often go 6/8. And that's it.\nWould more volume have lowered his numbers? Maybe, but I doubt it.\nAlso, very few players increase their stats in the playoffs. Reggie always did.\n\nSo let me start by saying I love Reggie miller. He was so entertaining. An absolutely bonkers clutch shooter and magical at times.\nThat being said while im sure the numbers are correct, Reggie just isn't that great of a number 1. He never really created his own shot. He had a terrifically balanced team that made teams focus on everyone and not just focus on stopping Reggie.\nI look at him as a slightly better version of Klay Thompson who was also much more charismatic and magical.\n\nHe is also one of the worst announcers that somehow keeps getting work\n\nDo we have numbers when excluding the shorter 3pt line?\n6th most valuable guard. Don't forget Dwade was the only reason Miami has ANY rings. Hes the second, or third best 2 guard in history, depending on how you value Kobe.", "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\n---\n\n[supprimé]\n\nOverall-Palpitation6·-10j·Modifié il y a-10j\nHe barely averaged 20 a game most years. He's like if Klay Thompson happened to be the Warriors' first option, on the same number of shot attempts.\n\ntrojan_man16·-10j\nGuy's prime was in the late 90s/early 2000s. That's the modern NBA's dead ball era. Even 18ppg was a big deal then, 20+ was actually impressive. With today's pace and a system optimizing his skills Reggie would be a 25ppg+ guy.\n\nMadpsu444·-10j\nReggie Miller is the most efficient first option in NBA playoff history\n\n---\n\nOverall-Palpitation6·-10j·Modifié il y a -10j\nFair enough, but even in his era, there were still 25-30ppg guys, and he was never one of them. Reggie finished top 10 in ppg once during his career, in 1989-90, when he finished 8th with 24.6ppg. Reggie never topped 26 USG%, and hovered in the low-to-mid 20s in USG% for his entire prime, so even if he was Indiana's de-facto #1 scorer, he really never got used or scored like a true #1, even in a lower possession era.\n\nvmpafq·-10j\nThat's cap. MJ, Shaq, Iverson types were averaging 30 then.", '[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\npacific_plywood · -10j\nWild to think that he\'s only a 5-time all star. Less than Kyle Lowry or Joe Johnson.\n\nBoogerSugarSovereign · -10j\nGuard was a stacked position in the East and Reggie\'s usage was a lot lower in the regular season than the playoffs. His highest regular season average FGA was 15.4. He has 8 playoff runs with a higher average FGA topping out at 22.5 in the 2000 Finals run.\n\nsmez86·-10j\nnot just "guard" either. you have to remember that rosters were constructed by position. sg1 in the east was guaranteed mj, so you only had 1 or 2 other spots.\n\npokexchespin·-10j\nwere they really? i wasn\'t around in the 90s, but i know when i started watching it was guards, forwards, and centers, same as all nba\n\nparrothead32812 ·-10j\n\nRyyKarsch · -10j\nThis is (mostly) true. He\'s not a sixth time all-star if he plays in the west, but he would have made it in 2016 and possibly the following season.\nHe was one of the best pure PGs in the league on one of the better regular season teams for nearly eight straight seasons. If Conley got one, then Lowry would have "sniffed" one, Imao.', "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nThe Pacers made 5 ECF in 7 seasons with Reggie Miller as their best player. That's a lot of winning.\nYou want to downgrade him because his team lost to the Shaq-Kobe Lakers in the Finals, or a super tight series to Jordan's Bulls in 7 games?\n\nReggie was an excellent player on an excellent team. I don't seek to downgrade him. I think he's properly rated on all-time lists and whatever. I am against his elevation to a status that he didn't actually play to in his career. In large part, the efficiency that you see here is the product of Reggie's very limited shot-making arsenal. The guy wasn't nearly as versatile a scorer as players like Jordan, Kobe and Bird who handled the ball much more, made plays for others as well as themselves, drove the ball, played through contact, etc., none of which Reggie had the physicality to do. Even compared to Steph, Reggie was a much, much more circumscribed scorer.\n\nNumber of points matters.\nSmaller sample sizes, no games played outside of peak/prime, etc.\nIf you pick MJ's best 2972 point stretch, I bet he clears Reggie easily."]</t>
+          <t>["[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nLakers team is pretty flawed and they're exploiting them well. With Wolves the question is still if they're a tier below. Obviously OkC is a tough matchup for anyone but I don't think Wolves have proved anything they didn't show last year.\n\nTimberwolves have beat OKC 2 times this season btw\n\nFor me it's less the teams and more so players.\nPaolo is the big standout for me\n\nMagic need to get some competent offensive players, particularly some shooters, around him and Franz this offseason.\n\nthat it has not panned out with him\nYes, Iwould be excited to see whatkind of numbers Paolo could put up if hehad more creation and shooting.\nHell, I would be excited to see what Paolo's numbers look like if the Magic were just ONE of the slowest pace team and just ONE of the lowest scoring teams and not dead last in both.\nI wonder what he would average if the Magic were 25th in pace and 25th in scoring versus 30th.", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nI would say the Twolves.I hadn't watched them much this season but their offense just looks so much better than last year. Ant seems to trust his teammates a lot more (obviously helps when they are making shots) and they aren't completely reliant on him playing iso in the end of games\n\nmajority of his attempts from dribble pull-ups. He was good in this area before but now he's elite and it's obviously a vital component to closing out games and stifling runs.\n\nJaden has taken an incremental step on offense, becoming much more willing/able to dribble-drive into short range pull-ups and attempts at the rim. Again, he would do this last season but now he's doing it with greater consistency.\n\nDonte as a bench creator/ball-handler who can hold his own somewhat on defense is a huge addition that helps mitigate Conley having down streaks.", '[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nDonte as a bench creator/ball-handler who can hold his own somewhat on defense is a huge addition that helps mitigate Conley having down streaks.\n\nJulius is less a dynamic scorer compared to KAT but he still flls the role as a "get-a-bucket" iso guy. He\'s also a better passer off the dribble although that hasn\'t been as apparent in this series so far.\n\nYeah I know Donte hasn\'t played well this series but I thought a guy like that to come off the bench and at least take some pressure off is definitely something they were missing last year\n\nI definitely thought the Wolves trading Kat was a huge downgrade but they definitely have adjusted to the new roster and look as good as ever.\n\nIndiana but I kind of expected it. I really think they have a legit shot against the Cavs next round. Their offense is no joke.\nWho are teams in the playoffs that have impressed you ? : r/nba\n\nWho are teams in the playoffs that have impressed you ? : r/nba', "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nIndiana and Minnesota to me\n\nPistons for me. Not surprised, just impressed with them\n\nWolves\nWolves are not surprising if you had watched them, I had picked them to beat the Lakers in six and\nwas specifically the team I wanted to dodge in the first round the most.\nThe have the highest ceiling of all the teams outside of Okc because they can be both elite offensively\nand defensively. Their only real flaw is decision making at times, but even then Ant has improved\nhugely on that end.\nI think they were ultimately under estimated as too many crowned the Lakers as being better than\nthey are actually are. Especially after the OKC H2Hs where their shooting output just wasn't very\nrealistic of who they were in a Playoff setting.\nI think the next best team is the Clippers, but man they have definitely found ways to lose games\nagainst the Nuggets.\nBut ultimately think it's going to end up pretty comfortably a OKC-MiN WCF and that is going to be\nan insane series.", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nI'm not responsible for the takes of others. I'm not anti-physicality but I am a fan of talent\nand skill in the game. Orlando and Houston have very little.\nBoth teams are hilariously overmatched in terms of shooting and scoring ability and have\nresorted to cheap shots and fouls to hurt their opponents instead of actually winning with\ntheir game. I'm not going to reward or applaud that behavior, it's not some equalizing skill to try to injure your opponents. Goons like Anthony Mason and Bill Laimbeer were bad for the game and I would've said as much at the time.\n\nMagic have no shooters. It's like watching the early 2000s. I don't mind it, but they won't win without a 3 ball.\n\nI'm sorry, but you're impressed with... The Magic?\nAnyway, I hate it but I gotta give credit to Indiana. They impressed me last year too and honestly, that offense is capable of beating literally everyone lol. not saying they're gonna win it all or anything, but Carlisle and the players deserve massive credit"]</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>D'après les discussions et analyses partagées dans les sources, Reggie Miller a été sélectionné **5 fois** pour le NBA All-Star Game au cours de sa carrière.
-*(Source : "Wild to think that he's only a 5-time all star." - Pacific_plywood, Score: 81.0%)*</t>
+          <t>Paolo Banchero et Franz Wagner.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D'apres les commentaires, Regie Miller a été 5 fois All-Star.</t>
+          <t>Paolo Banchero et Franz Wagner.</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8931386439238614</v>
+        <v>0.7130747467910522</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1111111111</v>
+        <v>0.9999999999</v>
       </c>
       <c r="H9" t="n">
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7293444238231716</v>
+        <v>0.9999917981944987</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -881,40 +862,42 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>D'après le thread Reddit sur l'avantage du terrain en playoffs, une équipe a-t-elle déjà atteint les Finals NBA sans jamais avoir eu l'avantage du terrain lors des tours précédents (contrairement aux Oilers en NHL cette année-là) ?</t>
+          <t>Quelles équipes ont le plus impressionné lors des playoffs ?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>["[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n101 upvotes : 44 commentaires\nr/nba·il y a 11j\n[Smith] This is now reality. Thunder vs Pacers will be the first NBA Finals since the luxury tax has been in effect where neither team was a taxpayer for that season.\n\n11 k upvotes : 948 commentaires\nr/hockey · il y a 13j\nThe Oilers are the first Canadian team to have home-ice advantage in the Stanley Cup Finals since the 2011 Vancouver Canucks\n\n2,5 k upvotes : 226 commentaires\nr/nba·ilya 11j\nThe Knicks have now lost to a lower seed in 5 straight playoff appearances3 of those losses came against the Pacers.\n\n2,7 k upvotes : 274 commentaires\nr/nba · il y a 2 m.\nThis was an all time Great day of nba playoff basketball\n\n183 upvotes : 39 commentaires\nr/nba· il y a 2 a\nNBA team logos over time\n\n464 upvotes : 136 commentaires\nWhich NBA team did not have home court advantage until the NBA Finals?\n\n113upvotes:80 commentaires\nr/nba • il y a 2 m.\nNBA Teams That Never Met in the Playoffs (Same Conference)\n\n8 upvotes : 20 commentaires\nr/nba • il y a 2 m.\nWho would've won the 2018 NBA Finals if the Rockets beat the Warriors in game 7 of the WCF?\n\n34 commentaires\nr/algeria ·il ya 9j\nAnyknownAlgerianbasketballteams?\n\n4 upvotes : 16 commentaires\nr/pacers ·il ya 28j\nIf Pacers and Nuggies Go to Finals, Who Has Homecourt?\n\n4 upvotes : 16 commentaires\nr/canes · il y a 1 m.\nThe last time we won a double OT game in the first round of the playoffs\n\n58 upvotes- 6 commentaires\nr/AllAmericanTV.il y a1a\nWhat NFL team will Spencer play for?", '[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n58 upvotes- 6 commentaires\nr/AllAmericanTV.il y a1a\nWhat NFL team will Spencer play for?\n\n25 upvotes : 19 commentaires\nr/nba · il y a 13 a\nNBA Court Explained\n\n25 upvotes : 19 commentaires\nr/nba· il ya6a\nCan someone explain to me what it means for a team in the playoffs to take home court?', '[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nO Repondre\nLadnil\nIt does prevent tanking. Just not 100% of it. But there are degrees of this\n\nO Répondre\nxelecunei\nI still think that the play-in is still a good idea. It just needs an overhaul.\nThey should just implement the play-in if the 7th and 8th seed is just 1-2 games ahead of the\n9th and 10th.\nIf the 7th seed is 4 or so games ahead, their spot should already be locked in. Same with the\n8th, if they are games ahead their spots should already be locked in.\nIt just doesn\'t make sense that an 8-game behind team having a shot at the play-offs.\n\nO Répondre\nelbosston\nIt\'s harder in basketball because usually the "better team" goes to the finals as basketball has less variance\nthan hockey due to how much harder it is to score in hockey\n\n\nsomeguy_3112\n2023 Heat Edit: just noticed that you asked for a team that had the home advantage in the finals. My bad', "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nO Repondre\nClownFundamentals · -11 j\nYeah, it'd really mess up their skates.\nO Repondre\nTeam_Ed·-11j\nNever in the NBA.\nThat's because Hockey is the favourite sport of the god of randomness and lower seeds win way more\noften than in basketball.\nThe NHL also has the same problem as the NBA of having the post-season be so much more intense that\nit's almost a different sport. What worked for a 110 point President's Trophy winner in the regular season\nmay not work at all in the playoffs.\nO Repondre\nareksoo ·-12j\nNever happened. For a team to make the final never having home court advantage you have to be the 5th\nseed. So the finals, needs a 6th or lower... but that's never happened because every finals contained at\nleast a 1st, 2nd or 3rd seed.\nO Repondre\nHeresTheAnswer\nyou could be any seed below 4th. If both teams were 8th seeds the one with better record would have\nhome court\nO Repondre\ndaymanahhhahhhhhh : -12 j\nThis has never happened in the nba.\nO Repondre\nSkinnecott · -12j\nif the lakers would have made the finals in 2023 it would have been heat vs lakers and only time heat had\nhomecourt would be finals. but denver beat them 3rd round and had homecourt over us\nO Repondre\nMaleficent_Resolve44 : -11 j\nHasn't happened yet. You'd need two proper low seeds to come out of both the west and east. Never\nbeen done before because the best teams usually get the highest seeds.\nO Repondre\nDr_Satan36·-12j\nsigto117·-12j", "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nalso gone ot the finals, like they did next year, the Suns would have been the lower seed each round until\nthe finals\nO Repondre\nTearz_in_rain ·-11j\nYou need to 8-5 seeds to make the finals for that to happen.\nWe've seen multiple teams get to the finals without home court at all, the most famous case likely being\nthe Rockets in 95, who won a title and had to beat the teams with the 4 best records in the league to do\nit.\nBut they never had home court at all.\nThe Knicks did it in the lock-out season in 99 and lost in the finals. The Heat I think did it twice with Jimmy\nButler.\nRépondre\nCapriciousManchild ·-12j\n2020 lakers and heat never had home court the entire playoffs for every game\nO Repondre\nSourBerry1425·-12j\n Comm. du top 1%\nDon't know off the top of my head but I bet this has happened to some Western Conference team when\nthe conferences were truly lopsided.\nO Repondre\npmurt007·-12j\nNever happened before. Lowest seed in the West to ever make it to the finals was the 1995 Rockets\nand they were 47-35\nO Repondre\nTheReturnOfTheOK·-12j\nAnd the defending champs.\nO Repondre\nHeresTheAnswer\nAnd had picked up Clyde Drexler in Feb\nO Repondre\nNever happened b/c the East's badness was vastly overexaggerated.\nO Repondre\nTurd_fergu50n ·-12j\nI'm not sure any hockey teams get home court tbh.\nO Repondre\nHeresTheAnswer\nHockey and MLB playoffs always seem like this\nO Repondre\nClownFundamentals · -11 j\nYeah, it'd really mess up their skates.\nO Repondre\nTeam_Ed·-11j\nNever in the NBA.", "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nbeen done before because the best teams usually get the highest seeds.\nO Repondre\nDr_Satan36·-12j\nsigto117·-12j\nWhy doesn't NBA hype up finals like Super Bowl? It should be a spectacle.\n422 upvotes : 38 commentaires\nr/nba·ilya 11j\nHas any team ever won anNBAtitleby winning4 Game7s?", "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nO Répondre\nsomeguy_3112\nYeah I missed that they asked for a team with home advantage in the finals, just edited my\ncomment\nDemonsReturns7 .-12j\nBut did they have home court adv in the finals though? I don't remember\nO Repondre\nhickok3 ·-12j\n Comm.du top 1%\nNo, Denver was the 1 seed iirc, and at the very least had home court.\nO Repondre\nrunevault · -11j\n Comm. du top 1%\nThe funny thing was the Nuggets took their foot off the gas after getting a 7 game lead over the 2\nseed Grizz and people worried they were throwing away home court in the finals because at least\nthe top 2 seeds in the east had better records.\nInstead Nuggets faced the Heat lol.\nO Répondre\nsomeguy_3112 · -12j\nYou're right, I missed the finals part in the post\nO Repondre\nYourWorstNightmare9·-12j\nThey would've had home court advantage in the Finals if the Lakers had beaten the Nuggets in the\nWCF that year.\nO Repondre\nwould really need a very lopsided difference between conference, like in 2008 when Golden State missed\nthe playoffs at 48-34 in the west but the Cavs could be a 5th seed at 45-37. That year, for example, had\nthe Suns and Rockets (both 55-27 and the 6th and 5th seed) made a run (not as crazy as it sounds, the\nLakers were 1st at only 57-25), with the Suns going to the finals, and the Magic (52-30) gotten hot and\nalso gone ot the finals, like they did next year, the Suns would have been the lower seed each round until\nthe finals\nO Repondre\nTearz_in_rain ·-11j", "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\n↑ 26 →O Répondre\n\n\nMayBeAGayBee\nThe main benefit of the play-in is just the fact that it can keep most of the teams hovering\naround that 6-seed/7-seed boundary in a death race until the very end of the regular season\nin order to avoid the play-in.Plus 7 and 8 seeds are basically freebie first round series\nanyways. It's not as if 1 and 2 seeds losing in the first round has ever been particularly\ncommon even before the play-in.\n\n\nUmmm https://www.basketball-reference.com/teams/MIA/2023.html\nNot a 9/10, but a play-in team that made it to the finals.\n\n\nO Répondre\nalmondsandrice69\nit only exists for an extra 4 games of revenue, but i would not mind if they reverted it to the\nsystem from the bubble, where it only kicked in if the teams were within a certain number of\ngames of each other. in 2024, 8-seed Miami won 7 more games than the 9-seed Bulls &amp; this\nyear, the grizzlies won 8 more games than the 9-seed kings. there's absolutely no reason why\neither of those teams needed to have a play-in game.\n\nO Repondre\nLadnil\nIt does prevent tanking. Just not 100% of it. But there are degrees of this", "[Contexte: Which NBA team did not have home court advantage until the NBA Finals? : r/nba]\nO Répondre\nMeece_\nAnd the argument that it prevents tanking falls somewhat short\nBefore the play ins, teams just gave up if they were like 5 or more games outside the 8 seed.\nNow damn near every teams fights for a play in spot or to keep themselves in the 6th seed or\nabove. It has revitalized the last third of the season.\nThen the play in games themselves are pretty fun too. Play ins have had nothing but positive\neffects for the NBA.\nThe chances of a 6-8th seed making the Finals is slim. Should we exlude them from the\nplayoffs entirely too? Feels silly to base things off their chances of making the Finals.\n\n\nO Répondre\njustmefishes\nThe play-in is worthwhile for its own sake. It's a few mini-Game 7s amongst not-great but not-\ncompletely-awful teams which makes for a nice appetizer going into the playoffs. Personally I\nfind it very interesting to see more flawed / average teams being put in that situation as you\nget to learn things about teams and players you otherwise wouldn't, because they'd either\nmiss the playoffs entirely or get bounced quickly in the first round by a much better team.\n\nre: the Mavs, I don't think they tanked, it was actually disastrous for them to miss the playoffs\nafter the Luka trade and it was almost entirely down to injuries. They got lucky in the lottery\nbut we know what their odds were, and it's really not worth tanking out of the play-in for such\nlow odds. A statistical fluke doesn't change that point.\n\n↑ 26 →O Répondre", "Which NBA team did not have home court advantage until the NBA Finals? : r/nba\n\nDonT012\nWhich NBA team did not have home court advantage until the NBA Finals?\nIn the NHL, the Edmonton Oilers just reached the NHL Finals. In their 3 rounds of play, they did not have home\nStars on the road.They will now host the Panthersat homeforthe Finals.\nWhich NBA team experienced this? First 3 rounds all on the road. Finals at home.\n\n\n← 272 →\n51\n\n\n\n\n\n\n55555_55555\nSix teams have made the Finals with lower than a 4 seed and none of them have had home court in the\nFinals. Think the answer is none, at least in the modern NBA.\n\n\nO Répondre\nrooftopworld\nGood lord, only 6? I knew it was rare, but I didn't think it was that rare.\n\n\n↑ 6S\nO Répondre\n\n\nSalty_Watermelon\nhttps://www.reddit.com/r/nba/comments/1066qq/which_nba_team_did_not_have_home_court_advantage/\n\n\nA 9th or 10th placed team is almost guaranteed to get smashed in the 1st round, and has pretty\nmuch no chance of making the Finals. It was cool that the 1Oth placed Heat made the playoffs\nuntil they lost to the Cavs in one of those most uncompetitive series of all time.\nAnd the argument that it prevents tanking falls somewhat short when the Mavericks have already\ntanked to avoid the play-in, and then got rewarded for it by keeping their pick and drafting\nLively..."]</t>
+          <t>["[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nIndiana and Minnesota to me\n\nPistons for me. Not surprised, just impressed with them\n\nWolves\nWolves are not surprising if you had watched them, I had picked them to beat the Lakers in six and\nwas specifically the team I wanted to dodge in the first round the most.\nThe have the highest ceiling of all the teams outside of Okc because they can be both elite offensively\nand defensively. Their only real flaw is decision making at times, but even then Ant has improved\nhugely on that end.\nI think they were ultimately under estimated as too many crowned the Lakers as being better than\nthey are actually are. Especially after the OKC H2Hs where their shooting output just wasn't very\nrealistic of who they were in a Playoff setting.\nI think the next best team is the Clippers, but man they have definitely found ways to lose games\nagainst the Nuggets.\nBut ultimately think it's going to end up pretty comfortably a OKC-MiN WCF and that is going to be\nan insane series.", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nIndiana but I kind of expected it. I really think they have a legit shot against the Cavs next round. Their offense is no joke.\nWho are teams in the playoffs that have impressed you ? : r/nba\n\nWho are teams in the playoffs that have impressed you ? : r/nba\n\nAnyone else feel like these playoffs are the most unpredictable in years?\n\nI think we should cherish the parity in the nba, because it's not going to last.", '[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nDonte as a bench creator/ball-handler who can hold his own somewhat on defense is a huge addition that helps mitigate Conley having down streaks.\n\nJulius is less a dynamic scorer compared to KAT but he still flls the role as a "get-a-bucket" iso guy. He\'s also a better passer off the dribble although that hasn\'t been as apparent in this series so far.\n\nYeah I know Donte hasn\'t played well this series but I thought a guy like that to come off the bench and at least take some pressure off is definitely something they were missing last year\n\nI definitely thought the Wolves trading Kat was a huge downgrade but they definitely have adjusted to the new roster and look as good as ever.\n\nIndiana but I kind of expected it. I really think they have a legit shot against the Cavs next round. Their offense is no joke.\nWho are teams in the playoffs that have impressed you ? : r/nba\n\nWho are teams in the playoffs that have impressed you ? : r/nba', "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nI would say the Twolves.I hadn't watched them much this season but their offense just looks so much better than last year. Ant seems to trust his teammates a lot more (obviously helps when they are making shots) and they aren't completely reliant on him playing iso in the end of games\n\nmajority of his attempts from dribble pull-ups. He was good in this area before but now he's elite and it's obviously a vital component to closing out games and stifling runs.\n\nJaden has taken an incremental step on offense, becoming much more willing/able to dribble-drive into short range pull-ups and attempts at the rim. Again, he would do this last season but now he's doing it with greater consistency.\n\nDonte as a bench creator/ball-handler who can hold his own somewhat on defense is a huge addition that helps mitigate Conley having down streaks.", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nPaolo and Cade both are mature difference makers. They look like they can carry on their shoulders.\n\npistons for sure. despite the crying about the whistle being too loose or too tight depending on the outcome, despite the knicks being incredibly healthy and the pistons being down ivey and now stew, they have been in every single game and cade is proving why he was the correct #1 pick in a draft that includes mobley, barnes, wagner, and sengun. once they are able to replace tobias (great signing for a stopgap veteran) through either trade, FA, or draft, they will be a top 5 team in the east for many years.\n\nI would say the Twolves.I hadn't watched them much this season but their offense just looks so much better than last year. Ant seems to trust his teammates a lot more (obviously helps when they are making shots) and they aren't completely reliant on him playing iso in the end of games"]</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>D'après les discussions Reddit analysées, **aucune équipe NBA n'a jamais atteint les Finales sans avoir eu l'avantage du terrain lors des tours précédents**. Plusieurs commentaires soulignent que cela n'est jamais arrivé dans l'histoire moderne de la NBA, notamment parce que les Finales opposent généralement au moins une équipe classée parmi les 3 premières de sa conférence (qui bénéficie donc de l'avantage du terrain).
-Les exemples cités comme les Rockets de 1995 (47-35, 6e de la Conférence Ouest) ou les Heat de 2023 (entrés en play-in) ont bien atteint les Finales, mais **ils avaient l'avantage du terrain en Finales** (car leur adversaire avait un meilleur bilan ou était mieux classé). Le seul cas où une équipe a *presque* vécu cette situation est celui des Lakers en 2023 : s'ils avaient battu Denver en demi-finale de Conférence, ils auraient eu l'avantage du terrain en Finales contre Miami (qui avait un bilan moins bon). Mais Denver, en tant que 1er de la Conférence, avait déjà l'avantage du terrain en Finales.
-**Réponse finale** : Non, une telle situation n'a jamais eu lieu en NBA. Les Finales nécessitent au moins une équipe avec un avantage du terrain (généralement les 3 premières têtes de série).</t>
+          <t>Les équipes qui ont le plus impressionné lors des playoffs 2024-25 selon les fans sont :
+- **Minnesota Timberwolves** : Leur progression offensive est remarquée, avec une meilleure confiance d'Ant (Anthony Edwards) envers ses coéquipiers et une attaque moins dépendante des iso. Leur potentiel défensif et offensif en fait une équipe redoutable, avec une série en demi-finale de conférence très attendue contre Oklahoma City.
+- **Indiana Pacers** : Leur attaque est saluée comme "no joke", et ils sont considérés comme un sérieux prétendant face aux Cavaliers en demi-finale de conférence Est.
+- **Detroit Pistons** : Malgré des blessures (Ivey, Stewart), Cade Cunningham confirme son statut de leader, et l'équipe reste compétitive, avec un projet prometteur pour les années à venir.
+*Source : Retours de fans sur Reddit (saison 2024-25).*</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Non. Selon les commentaires du thread, ce scénario ne s'est jamais produit en NBA. Le cas le plus proche reste les Houston Rockets de 1995, qui ont remporté le titre sans avoir l'avantage du terrain à aucun moment des playoffs, mais aucune équipe n'a atteint les Finals dans cette configuration exacte (contrairement à la NHL, où les Oilers l'ont fait la même année selon le post).</t>
+          <t>D'apres les commentaires, les équipes les plus impressionnants sont les Wolwes (Minnesota), les Indiana Pacers et les Pistons (Detroit).</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.7857142857142857</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F10" t="n">
-        <v>0.950827731289956</v>
+        <v>0.8309572517660736</v>
       </c>
       <c r="G10" t="n">
-        <v>0.8412257495497359</v>
+        <v>0.8333333332916666</v>
       </c>
       <c r="H10" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6027034278868613</v>
+        <v>0.5400155759402114</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -930,42 +913,48 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Selon l'auteur du post 'Who are teams in the playoffs that have impressed you?', quel duo de jeunes ailiers du Magic cite-t-il comme son duo préféré de la ligue ?</t>
+          <t>En quoi les fans considerent Randle comme une révélation cette saison?</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>["[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nxWolfsbane : -1 m.\nMagic have no shooters. It's like watching the early 2000s. I don't mind it, but they won't win\nwithout a 3 ball.\n\nARGHETH · -1 m.\n\njustletmeregisteryou · -1 m.\n+Auteur-ricetop1%\nI'm sorry, but you're impressed with... The Magic?\nAnyway, I hate it but I gotta give credit to Indiana. They impressed me last year too ad honestly, that\noffense is capable of beating literally everyone lol. not saying they're gonna win it all or anything, but\nCarlisle and the players deserve massive credit\n\n←\n\nKlumber · -1 m.\nRespect. I will always wonder 'what if' about last year's run without Giannis, but this year I think the\ndifference is there.\n\nMannerSuperb AO . -1 m.\nPaolo and Franz have been a dynamic wing duo this whole series agaisnt one of the best defensive\nteams in basketball plus the defending champs. Yes the supporting cast has been laughably bad at\ntimes around them offensively but they guard their asses off and really giving the Celtics a fight\ndespite missing Suggs and the other Wagner brother. I thkkk their floor spacers and average PG away\nfrom being an true contender\n\ngeorgiosauce : -1 m.\nMagic are down 3-1 despite injuring 3 Celtics starters along the way, they're solid trash\n\nPeachTreeDish91 · -1 m.\nYou really seem like the type of dude who spends 10 minutes watching the youtube highlights\nwhile checking the box score, then spends the next 60 minutes typing bs out the ass on reddit", '[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nKingmav24 · -1 m.\nthis might be the least watched finals of all time\n\nDeep down they all still want a Celtics-Lakers final\n\ndelta_velorum : -1 m.\nIf it\'s a Wolves-Pacers final, I\'m switching to watching the WNBA\n\nsmkmn13.-1 m.\nRandle shooting 45% from three is a massive boost for a 33% career guy. Balancing out\nDonte/NAW/Copley\'s rough shooting.\n\nRandomerThanYours·-1m.\nMagic have been solid but I wouldn\'t really call it taking us to the brink. Atlanta a couple years ago was\nthe real scary first round.\n\nBoneslIX · -1 m.\nMagic is one of those "if they figure it out, they\'re gonna be scary" examples. I\'ve been pretty high on\nthem for 2+ seasons. Hoping for health for them next year. They will be a regular conference\ncontender if they get a little more 3pt shooting and continue to ride the growth of Paolo and the\nWagners.\n\n[supprimé] · -1 m.\nBut with the magic you\'re always moments away from a serious injury\n\nSteamingHotChocolate·-1 m.\nthis series is certainly taking me to the brink of insanity for that reason yeah\n\nEasy_Magician_925 ·-1 m.\nhl Magic have been down 2 of their more impactful players all series and could easily be tied 2-2 let\nalone up 3-1.\n\nhollow-ataraxia·-1m.\nTrae won\'t get credit for it because he went cold in the second half of game 6 and he started the\nseries slow but that game 5 and first half of game 6 was some of the best basketball I\'ve ever seen\nhim play. He single handedly almost willed us to a game 7 but ran out of gas.', '[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\n2. Jaden has taken an incremental step on offense, becoming much more willing/able to dribble-drive into short range pull-ups and attempts at the rim. Again, he would do this last season but now he\'s doing it with greater consistency.\n\n3. Donte as a bench creator/ball-handler who can hold his own somewhat on defense is a huge addition that helps mitigate Conley having down streaks.\n\n4. Julius is less a dynamic scorer compared to KAT but he still flls the role as a "get-a-bucket" iso guy. He\'s also a better passer off the dribble although that hasn\'t been as apparent in this series so far.\n\nYeah I know Donte hasn\'t played well this series but I thought a guy like that to come off the bench and at least take some pressure off is definitely something they were missing last year\n\nI definitely thought the Wolves trading Kat was a huge downgrade but they definitely have adjusted to the new roster and look as good as ever.\n\nIndiana but I kind of expected it. I really think they have a legit shot against the Cavs next round. Their offense is no joke.\nWho are teams in the playoffs that have impressed you ? : r/nba\n\nSe connecter\n\nWho are teams in the playoffs that have impressed you ? : r/nba\n\nAnyone else feel like these playoffs are the most unpredictable in years?\n\nI think we should cherish the parity in the nba, because it\'s not going to last.', "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nthat it has not panned out with him\nYes, Iwould be excited to see whatkind of numbers Paolo could put up if hehad more creation and shooting.\nHell, I would be excited to see what Paolo's numbers look like if the Magic were just ONE of the slowest pace team and just ONE of the lowest scoring teams and not dead last in both.\nI wonder what he would average if the Magic were 25th in pace and 25th in scoring versus 30th.\n\nPaolo and Cade both are mature difference makers. They look like they can carry on their shoulders.\n\npistons for sure. despite the crying about the whistle being too loose or too tight depending on the outcome, despite the knicks being incredibly healthy and the pistons being down ivey and now stew, they have been in every single game and cade is proving why he was the correct #1 pick in a draft that includes mobley, barnes, wagner, and sengun. once they are able to replace tobias (great signing for a stopgap veteran) through either trade, FA, or draft, they will be a top 5 team in the east for many years.\n\nI would say the Twolves.I hadn't watched them much this season but their offense just looks so much better than last year. Ant seems to trust his teammates a lot more (obviously helps when they are making shots) and they aren't completely reliant on him playing iso in the end of games\n\nmajority of his attempts from dribble pull-ups. He was good in this area before but now he's elite and it's obviously a vital component to closing out games and stifling runs.", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\ninshamblesx · -1 m.\nwolves by a mile\n\nTemperedTorture · -1 m.\nWolves by far. Particularly Edwards. I hadn't seen any Wolves games going into the playoffs, so I had no\nclue just how amazing Edwards was and he's really in the middle of a massive leap these playoffs. They\nhave a strong team -- and that's important these playoffs more than ever. Hero/iso ball is essentially dead\nbecause of how good defences have gotten.\nIt's been a joy to watch the Lakers/Wolves series and I'm becoming a huge fan of Ant. OKC, Celts and Cavs\nare performing up to expectation. Kinda always knew that Gsw would muscle through because of their\nsheer playoff and championship experience. Wasn't expecting the way Wolves have torn into the Lakers\nand exposed their lack of roster depth.\n\nOther-Owl4441\nLakers team is pretty flawed and they're exploiting them well. With Wolves the question is still if\nthey're a tier below. Obviously OkC is a tough matchup for anyone but I don't think Wolves have\nproved anything they didn't show last year.\n\nBrofessor-\nTimberwolves have beat OKC 2 times this season btw\n\nNiceguydan8 · -1 m.\nFor me it's less the teams and more so players.\nPaolo is the big standout for me\n\nProof-Umpire-7718\nAuteur-rice top 1%\nMagic need to get some competent offensive playsrs, particularly some shooters, around him and\nFranz this offseason.", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nTallnFrosty · -1 m.\nuntil franz fixes his shooting, i don't think 'dynamic' is the right word for him\n\nlegendofthededbug · -1 m.\nthepeachgod . -1 m.\nIndiana is gonna have a better chance at beating Cleveland than people will give them\n\nSiakam is themost underrated playerin the league as far as impact towards winning.if that team's\nclicking, which they seem to be with Hali dishing the way he is right now, they're a tough out for\nanyone\n\nshhhhhhhwish · -1 m.\nBy far the toughest series last year for the Celtics. I think we'll get a Celtics Indy rematch tbh... no one\nwill see it coming but it wasn't a fluke Indy got there last year\n\nYankeeknickfan · -1 m.\nIt's impressive that they're finally not just scraping by a team that's injured and straight up\nDominating a worse team. Definitely better than last year\nBut the bucks are awful. Really don't get why dominating them says anything about Cleveland\n\nPistons are one shot creator from being an ECF contending team imo.\n\nMannerSuperb Ao\nbefore his injury\n\naenima1991 : -1 m.\n10000% I keep thinking that - where would they be w Ivey. Probably up in this series.\n\nOther-Owl4441 : -1 m.\nLove Ivey but isn't the ideal profile for that missing piece a shot creator who's a knockdown\nshooter, instead?\n\nPootieTooGood\nI'm praying that they do not believe Ty Jerome is their answer since they're the team with the cap\nspace to pry him away from us\n\ninshamblesx · -1 m.\nwolves by a mile", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nNo_Albatross916 . -1 m.\nIndiana and Minnesota to me\n\n57\n\nthereticent · -1 m.\nPistons for me. Not surprised, just impressed with them\n\nProof-Umpire-7718 · -1 m.\nWolves\n\n61\nWolves are not surprising if you had watched them, I had picked them to beat the Lakers in six and\nwas specifically the team I wanted to dodge in the first round the most.\nThe have the highest ceiling of all the teams outside of Okc because they can be both elite offensively\nand defensively. Their only real flaw is decision making at times, but even then Ant has improved\nhugely on that end.\nI think they were ultimately under estimated as too many crowned the Lakers as being better than\nthey are actually are. Especially after the OKC H2Hs where their shooting output just wasn't very\nrealistic of who they were in a Playoff setting.\nI think the next best team is the Clippers, but man they have definitely found ways to lose games\nagainst the Nuggets.\nBut ultimately think it's going to end up pretty comfortably a OKC-MiN WCF and that is going to be\nan insane series.\n\nMaybe to you but we got humbled last year\n\nCade. Dude needs to seriously cut down on the turnovers, but he's a bucket.\n\nI get frustrated with his sloppy turnovers a lot but he's kind of in the position he has to. Too many possessions where\nwe can't even get the ball inside 30 feet of the basket if he doesn't touch the ball", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nCade has really impressed with his play but even more so with his leadership. I think Detroid has a\nmaturity and emotion problem which can be buffed out with age and experience. He's holding both\nhimself and his teammates accountable. Him pushing his rookie away yesterday to keep him in check,\nchill him out and stop him from getting a stupid tech was some real shit.\n\nIt's a talent issue. Stew and Holland definitely run hot but that's not the issue. The team feeds off that a lot of times. They just don't have a secondary scoring\noption outside of Cade especially with Ivey hurt. A lot of this is being passed on to Dennis\nSchroeder/Malik Beasley/Tobias Harris which is a good patch job for this season but it's not\nreliable or what you want in a playoff series.\n\nHe also needs to seriously work on his jumper. His 3-ball isn't very good. That needs to be\nnorth of 35% to explode.\n\nWas north of 35% this season.\n\nthey don't really have a secondary playmaker. Their second best shot creator\nShroeder. He's being asked to do a lot as the sole focus of the opposing team.\n\nYou must hate good offense, I have been disgusted watching the Magic play\n\nGood offense is a lot harder to come by in playoff basketball tho. Games are more physical and lower\nscoring. Warriors have a great offense and struggling against a physical rockets defense\n\nTheMagicoffenseisbasketballterrorism.", "Who are teams in the playoffs that have impressed you ? : r/nba\n\nMannerSuperb\nWho are teams in the playoffs that have impressed you ?\nFor me it's the magic. Despite awful shooting , they have really taken the defending champs to the brink. I'm a\nlittle biased as a Duke fan but Paolo and Franz are absolute dogs and my favorite young wing duo in the\nleague those guys have shown they are built for playoff basketball with their shot making ability and\ncompeting defensively. I truly hope orl can get those kids some real shooters and a true point guard theirs\nanother level their games and overall team can reach if they simply had some floor spacing and average guard\nplay around them.\n\n31\n236\n\nNotWD . -1 m.\nAnt's been a machine as expected, but Randle's genuinely beating the beyblade allegations and it's so\nnice to see\n\n186\n\nMG_MN .-1 m.\nRandle has been a revelation. His bully ball has worked perfectly on offense, and his physically is a big\nreason LeBron has run out of gas\n\n55\n\nGbaby245 : -1 m.\nRandle knows he can out muscle most guys one on one, and then makes the correct read when\ndoubles come. He also plays defense with his chest, not hands so he doesn't get the fouls Kat did.\nLuka and Bron can't just shove Randle out of the way on every drive.\n\n32", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nTheMagicoffenseisbasketballterrorism.\n\nThe Magic and Rockets are football teams effectively just roughing up their superior opponents\nand injuring them. In fact the only reason either team won a game is due to taking out the elite\nplayers on Boston/GS.\nI am not impressed in the slightest. It's bush league stuff due to a complete lack of skill on both\nrosters.\n\nThat's going a little overboard\n\nAm I wrong though\n\nThat's on the officials more than the teams. If the refs are swallowing their whistles and letting\na team play ultra physical they're going to continue to play that way until they start racking up\nfouls. I truly don't get some of the ppl complaining about the physicality of teams on this sub\nyou can't have it both ways. This sub had stretches of complaining about how soft the game\nhas gotten and then when refs are allowing teams to play more physical then their playing\nfootball\n\nI'm not responsible for the takes of others. I'm not anti-physicality but I am a fan of talent\nand skill in the game. Orlando and Houston have very little.\nBoth teams are hilariously overmatched in terms of shooting and scoring ability and have\nresorted to cheap shots and fouls to hurt their opponents instead of actually winning with\ntheir game. I'm not going to reward or applaud that behavior, it's not some equalizing skill\nto try to injure your opponents. Goons like Anthony Mason and Bill Laimbeer were bad for\nthe game and I would've said as much at the time."]</t>
+          <t>["[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\n31\n236\n\nAnt's been a machine as expected, but Randle's genuinely beating the beyblade allegations and it's so nice to see\n\n186\n\nRandle has been a revelation. His bully ball has worked perfectly on offense, and his physically is a big reason LeBron has run out of gas\n\n55\n\nRandle knows he can out muscle most guys one on one, and then makes the correct read when doubles come. He also plays defense with his chest, not hands so he doesn't get the fouls Kat did. Luka and Bron can't just shove Randle out of the way on every drive.\n\n32\n\nYou knew when I KNEW it would work? When Rashad McCants co-signed it.\nThe biggest revelation to me has been Randle's commitment on the defensive end. He looks much more engaged and focused right now. I'm hoping he won't stay as interested in the second round (if he beats his former team and if the Warriors beat the Rockets).", "[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\nRandle has been past beyblade mode for years now, unfortunately he's been hurt the last few times the Knicks were in the playoffs and everyone was watching so people still think he's the Randle from 4-5 years ago\n\n36\n\nRandle's playoff reputation really ignores the circumstances. He had 1 actual poor playoff series against the Hawks, with 3 million year old DRose as the next best player on the roster, and then had like 3 ankle sprains in 2 weeks the next time the Knicks made the playoffs. This is really his first opportunity to shine, and it's been fun to watch him and donte in these playoffs on another team.\n\nHoping we get T-wolves vs Pacers in the finals so we get some real beyblade duel action\n\n31\n\nWhat's the beyblade joke I don't get it\n\nBoth Randle and Siakam used to spam spin moves every time they went to the basket\n\nAhh haha\n\nthis might be the least watched finals of all time\n\nDeep down they all still want a Celtics-Lakers final", '[Contexte: How is it that the two best teams in the playoffs based on stats, having a chance of playing against each other in the Finals, is considered to be a snoozefest?]\nO Repondre\n\nhoppergym ·-15j\nWho considers it to be a snooze fest? Please cite Sources\n\nO Repondre\n\ncody_d_baker ·-15j\nAgreed, I\'m tired of this narrative on r/nba, all I\'m seeing is constant excitement over the small market\nteams and people saying the ratings don\'t matter\nO Repondre\n\nDelusional_Donut ·-15j\nIthink it\'s carry-overdiscoursefromlastyear\'s playoffs,casual social media sports content creators\nwho don\'t actually watch the sport just saying whatever so they can post 3 YouTube shorts a day\nO Repondre\n\nhoppergym ·-14j\nWho? What nba media? That\'s all I\'m asking.\nO Repondre\n\nTerrible_Shelter_345·-15j\nIt\'s probably just salty Celtics fans, Knicks fans, Jokic stans, and Ant stans all bitching online\nNo one in real life would ever be talking "tv ratings" at the bar or the kickback watching a ball game\nImao\n个 2\nRepondre', "[Contexte: Reggie Miller is the most efficient first option in NBA playoff history : r/nba]\nO Repondre\nNYC had a pretty egalitarian offence with Spree and LJ both getting a decent share of the shots.\nPeople look at Reggie's game as being more modern and overrate him a bunch. He's basically Klay Thompson without the defense (and honestly he didn't really seem to have the explosive scoring potential that Klay had, although that may be due to Klay facing weaker defense playing with multiple HoF players).", '[Contexte: Who are teams in the playoffs that have impressed you ? : r/nba]\n31\n\nWhat\'s the beyblade joke I don\'t get it\n\nBoth Randle and Siakam used to spam spin moves every time they went to the basket\n\nAhh haha\n\nthis might be the least watched finals of all time\n\nDeep down they all still want a Celtics-Lakers final\n\nIf it\'s a Wolves-Pacers final, I\'m switching to watching the WNBA\n\nRandle shooting 45% from three is a massive boost for a 33% career guy. Balancing out Donte/NAW/Copley\'s rough shooting.\n\nMagic have been solid but I wouldn\'t really call it taking us to the brink. Atlanta a couple years ago was the real scary first round.\n\nMagic is one of those "if they figure it out, they\'re gonna be scary" examples. I\'ve been pretty high on them for 2+ seasons. Hoping for health for them next year. They will be a regular conference contender if they get a little more 3pt shooting and continue to ride the growth of Paolo and the Wagners.\n\nBut with the magic you\'re always moments away from a serious injury']</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>D'après le contexte fourni, le duo de jeunes ailiers du Magic cité comme son duo préféré de la ligue par l'auteur du post est **Paolo Banchero et Franz Wagner**.</t>
+          <t>Les fans considèrent Randle comme une révélation cette saison pour plusieurs raisons clés :
+1. **Performances offensives dominantes** : Son jeu physique et son "bully ball" (style de jeu agressif) ont parfaitement fonctionné, lui permettant de dominer les défenses. Il a notamment prouvé qu'il pouvait tenir tête à des joueurs comme LeBron James en matchup direct, ce qui était impensable auparavant.
+2. **Amélioration défensive** : Randle a surpris par son engagement accru en défense, jouant avec sa poitrine plutôt qu'avec les mains pour éviter les fautes, contrairement à ses anciennes critiques sur ce point.
+3. **Efficacité à trois points** : Avec un pourcentage de 45% à trois points cette saison (contre 33% en carrière), il a ajouté une dimension nouvelle à son jeu, équilibrant les lacunes de ses coéquipiers.
+4. **Contexte historique** : Après des années de blessures et de doutes (notamment à cause de son image de "beyblade" due à ses spin moves), cette saison marque sa première réelle opportunité de briller en playoffs sans être freiné par des problèmes physiques.
+5. **Impact sur les adversaires** : Son jeu physique a épuisé des stars comme LeBron, montrant qu'il peut rivaliser avec les meilleurs sans se faire dominer physiquement.
+En résumé, Randle a transformé son image de joueur inconstant en leader dominant, justifiant pleinement son statut de révélation.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Paolo (Banchero) et Franz (Wagner)</t>
+          <t>Principalement à cause de son impact physique sur le jeu, son bully ball, ses spin moves, son implication défensive et sa meilleure efficacité à 3pts.</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.9440630071529478</v>
+        <v>0.945827297339735</v>
       </c>
       <c r="G11" t="n">
-        <v>0.7511904761797449</v>
+        <v>0.8666666666377778</v>
       </c>
       <c r="H11" t="n">
         <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>0.9616402700344528</v>
+        <v>0.8690660132585237</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>bruitee</t>
+          <t>bruitée</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">

</xml_diff>